<commit_message>
Finaliza cambios de SASISOPA - faltante 2
</commit_message>
<xml_diff>
--- a/sasisopa-machotes/sasisopa-machotes/F-02-02_Matriz_de_Identificación_de_Aspectos_e_Impactos_Ambientales.xlsx
+++ b/sasisopa-machotes/sasisopa-machotes/F-02-02_Matriz_de_Identificación_de_Aspectos_e_Impactos_Ambientales.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30228"/>
   <workbookPr codeName="ThisWorkbook" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Denisse Gutierrez\Desktop\GESTORIA\SASISOPA\MACHOTE SASISOPA ACTUALIZADO\2. ASPECTOS AMBIENTALES PELIGROS Y RIESGOS\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/01dae4c2401b18f1/Escritorio/portal-tecnocontrol-main GIt/portal-tecnocontrol/sasisopa-machotes/sasisopa-machotes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{511E3075-E7BB-4278-9A7A-1E44DF908B4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{511E3075-E7BB-4278-9A7A-1E44DF908B4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{31C79D52-B758-4EB3-935E-C3DEF4D84079}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ANEXO 1" sheetId="2" r:id="rId1"/>
@@ -1328,12 +1328,105 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1352,102 +1445,6 @@
     <xf numFmtId="0" fontId="7" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="13" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
@@ -1458,6 +1455,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2978,37 +2978,37 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Hoja2"/>
   <dimension ref="A1:D26"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.88671875" defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="6.109375" style="4" customWidth="1"/>
-    <col min="2" max="2" width="8.33203125" style="4" customWidth="1"/>
+    <col min="1" max="1" width="6.140625" style="4" customWidth="1"/>
+    <col min="2" max="2" width="8.28515625" style="4" customWidth="1"/>
     <col min="3" max="3" width="13" style="4" customWidth="1"/>
-    <col min="4" max="4" width="63.33203125" style="4" customWidth="1"/>
-    <col min="5" max="16384" width="10.88671875" style="4"/>
+    <col min="4" max="4" width="63.28515625" style="4" customWidth="1"/>
+    <col min="5" max="16384" width="10.85546875" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="37" t="s">
+    <row r="1" spans="1:4" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="49" t="s">
         <v>93</v>
       </c>
-      <c r="B1" s="37"/>
-      <c r="C1" s="37"/>
-      <c r="D1" s="37"/>
-    </row>
-    <row r="2" spans="1:4" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="43" t="s">
+      <c r="B1" s="49"/>
+      <c r="C1" s="49"/>
+      <c r="D1" s="49"/>
+    </row>
+    <row r="2" spans="1:4" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="58" t="s">
         <v>27</v>
       </c>
       <c r="B2" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="C2" s="38" t="s">
+      <c r="C2" s="52" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="38"/>
-    </row>
-    <row r="3" spans="1:4" ht="41.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="43"/>
+      <c r="D2" s="52"/>
+    </row>
+    <row r="3" spans="1:4" ht="41.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="58"/>
       <c r="B3" s="1">
         <v>1</v>
       </c>
@@ -3019,8 +3019,8 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="42.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="43"/>
+    <row r="4" spans="1:4" ht="42.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="58"/>
       <c r="B4" s="1">
         <v>2</v>
       </c>
@@ -3031,8 +3031,8 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="41.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="43"/>
+    <row r="5" spans="1:4" ht="41.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="58"/>
       <c r="B5" s="1">
         <v>3</v>
       </c>
@@ -3043,18 +3043,18 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="43"/>
+    <row r="6" spans="1:4" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="58"/>
       <c r="B6" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="C6" s="38" t="s">
+      <c r="C6" s="52" t="s">
         <v>7</v>
       </c>
-      <c r="D6" s="38"/>
-    </row>
-    <row r="7" spans="1:4" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="43"/>
+      <c r="D6" s="52"/>
+    </row>
+    <row r="7" spans="1:4" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="58"/>
       <c r="B7" s="1">
         <v>1</v>
       </c>
@@ -3065,8 +3065,8 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="43"/>
+    <row r="8" spans="1:4" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="58"/>
       <c r="B8" s="1">
         <v>2</v>
       </c>
@@ -3077,8 +3077,8 @@
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="43"/>
+    <row r="9" spans="1:4" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="58"/>
       <c r="B9" s="1">
         <v>3</v>
       </c>
@@ -3089,18 +3089,18 @@
         <v>13</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="43"/>
+    <row r="10" spans="1:4" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="58"/>
       <c r="B10" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="C10" s="26" t="s">
+      <c r="C10" s="50" t="s">
         <v>14</v>
       </c>
-      <c r="D10" s="27"/>
-    </row>
-    <row r="11" spans="1:4" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="43"/>
+      <c r="D10" s="51"/>
+    </row>
+    <row r="11" spans="1:4" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="58"/>
       <c r="B11" s="1">
         <v>1</v>
       </c>
@@ -3111,8 +3111,8 @@
         <v>16</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="43"/>
+    <row r="12" spans="1:4" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="58"/>
       <c r="B12" s="1">
         <v>2</v>
       </c>
@@ -3123,8 +3123,8 @@
         <v>18</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="43"/>
+    <row r="13" spans="1:4" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="58"/>
       <c r="B13" s="1">
         <v>3</v>
       </c>
@@ -3135,114 +3135,118 @@
         <v>20</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B14" s="42"/>
-      <c r="C14" s="42"/>
-      <c r="D14" s="42"/>
-    </row>
-    <row r="15" spans="1:4" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="39" t="s">
+    <row r="14" spans="1:4" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B14" s="57"/>
+      <c r="C14" s="57"/>
+      <c r="D14" s="57"/>
+    </row>
+    <row r="15" spans="1:4" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="53" t="s">
         <v>28</v>
       </c>
       <c r="B15" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="C15" s="38" t="s">
+      <c r="C15" s="52" t="s">
         <v>68</v>
       </c>
-      <c r="D15" s="38"/>
-    </row>
-    <row r="16" spans="1:4" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="40"/>
+      <c r="D15" s="52"/>
+    </row>
+    <row r="16" spans="1:4" ht="19.899999999999999" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="54"/>
       <c r="B16" s="7">
         <v>0</v>
       </c>
-      <c r="C16" s="31" t="s">
+      <c r="C16" s="62" t="s">
         <v>22</v>
       </c>
-      <c r="D16" s="31"/>
-    </row>
-    <row r="17" spans="1:4" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="40"/>
+      <c r="D16" s="62"/>
+    </row>
+    <row r="17" spans="1:4" ht="19.899999999999999" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="54"/>
       <c r="B17" s="7">
         <v>10</v>
       </c>
-      <c r="C17" s="32" t="s">
+      <c r="C17" s="63" t="s">
         <v>23</v>
       </c>
-      <c r="D17" s="33"/>
-    </row>
-    <row r="18" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="40"/>
+      <c r="D17" s="64"/>
+    </row>
+    <row r="18" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="54"/>
       <c r="B18" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="C18" s="26" t="s">
+      <c r="C18" s="50" t="s">
         <v>52</v>
       </c>
-      <c r="D18" s="27"/>
-    </row>
-    <row r="19" spans="1:4" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="40"/>
+      <c r="D18" s="51"/>
+    </row>
+    <row r="19" spans="1:4" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="54"/>
       <c r="B19" s="7">
         <v>0</v>
       </c>
-      <c r="C19" s="34" t="s">
+      <c r="C19" s="56" t="s">
         <v>21</v>
       </c>
-      <c r="D19" s="34"/>
-    </row>
-    <row r="20" spans="1:4" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="41"/>
+      <c r="D19" s="56"/>
+    </row>
+    <row r="20" spans="1:4" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="55"/>
       <c r="B20" s="7">
         <v>10</v>
       </c>
-      <c r="C20" s="34" t="s">
+      <c r="C20" s="56" t="s">
         <v>30</v>
       </c>
-      <c r="D20" s="34"/>
-    </row>
-    <row r="22" spans="1:4" ht="14.4" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="23" spans="1:4" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="26" t="s">
+      <c r="D20" s="56"/>
+    </row>
+    <row r="22" spans="1:4" ht="13.5" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="23" spans="1:4" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="50" t="s">
         <v>77</v>
       </c>
-      <c r="B23" s="30"/>
-      <c r="C23" s="30"/>
-      <c r="D23" s="27"/>
-    </row>
-    <row r="24" spans="1:4" ht="73.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="26" t="s">
+      <c r="B23" s="61"/>
+      <c r="C23" s="61"/>
+      <c r="D23" s="51"/>
+    </row>
+    <row r="24" spans="1:4" ht="73.900000000000006" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="50" t="s">
         <v>25</v>
       </c>
-      <c r="B24" s="27"/>
-      <c r="C24" s="28" t="s">
+      <c r="B24" s="51"/>
+      <c r="C24" s="59" t="s">
         <v>73</v>
       </c>
-      <c r="D24" s="29"/>
-    </row>
-    <row r="25" spans="1:4" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="26" t="s">
+      <c r="D24" s="60"/>
+    </row>
+    <row r="25" spans="1:4" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="50" t="s">
         <v>26</v>
       </c>
-      <c r="B25" s="27"/>
-      <c r="C25" s="35" t="s">
+      <c r="B25" s="51"/>
+      <c r="C25" s="47" t="s">
         <v>74</v>
       </c>
-      <c r="D25" s="36"/>
-    </row>
-    <row r="26" spans="1:4" ht="44.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="26" t="s">
+      <c r="D25" s="48"/>
+    </row>
+    <row r="26" spans="1:4" ht="44.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="50" t="s">
         <v>24</v>
       </c>
-      <c r="B26" s="27"/>
-      <c r="C26" s="35" t="s">
+      <c r="B26" s="51"/>
+      <c r="C26" s="47" t="s">
         <v>72</v>
       </c>
-      <c r="D26" s="36"/>
+      <c r="D26" s="48"/>
     </row>
   </sheetData>
   <mergeCells count="20">
+    <mergeCell ref="C16:D16"/>
+    <mergeCell ref="C17:D17"/>
+    <mergeCell ref="C18:D18"/>
+    <mergeCell ref="C19:D19"/>
     <mergeCell ref="C26:D26"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A26:B26"/>
@@ -3259,10 +3263,6 @@
     <mergeCell ref="A25:B25"/>
     <mergeCell ref="C24:D24"/>
     <mergeCell ref="A23:D23"/>
-    <mergeCell ref="C16:D16"/>
-    <mergeCell ref="C17:D17"/>
-    <mergeCell ref="C18:D18"/>
-    <mergeCell ref="C19:D19"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1.0119047619047619" bottom="1" header="0.3" footer="0.3"/>
@@ -3285,137 +3285,137 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:W27"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.88671875" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="29.88671875" style="10" customWidth="1"/>
+    <col min="1" max="1" width="29.85546875" style="10" customWidth="1"/>
     <col min="2" max="3" width="7" style="10" customWidth="1"/>
     <col min="4" max="4" width="26" style="10" customWidth="1"/>
-    <col min="5" max="5" width="19.33203125" style="10" customWidth="1"/>
-    <col min="6" max="6" width="5.88671875" style="10" customWidth="1"/>
-    <col min="7" max="7" width="6.33203125" style="10" customWidth="1"/>
+    <col min="5" max="5" width="19.28515625" style="10" customWidth="1"/>
+    <col min="6" max="6" width="5.85546875" style="10" customWidth="1"/>
+    <col min="7" max="7" width="6.28515625" style="10" customWidth="1"/>
     <col min="8" max="8" width="6" style="10" customWidth="1"/>
-    <col min="9" max="9" width="6.44140625" style="10" customWidth="1"/>
-    <col min="10" max="17" width="5.44140625" style="10" customWidth="1"/>
-    <col min="18" max="18" width="4.33203125" style="10" customWidth="1"/>
+    <col min="9" max="9" width="6.42578125" style="10" customWidth="1"/>
+    <col min="10" max="17" width="5.42578125" style="10" customWidth="1"/>
+    <col min="18" max="18" width="4.28515625" style="10" customWidth="1"/>
     <col min="19" max="19" width="3" style="10" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="11.6640625" style="10" customWidth="1"/>
-    <col min="21" max="21" width="9.6640625" style="10" customWidth="1"/>
-    <col min="22" max="22" width="29.33203125" style="10" customWidth="1"/>
+    <col min="20" max="20" width="11.7109375" style="10" customWidth="1"/>
+    <col min="21" max="21" width="9.7109375" style="10" customWidth="1"/>
+    <col min="22" max="22" width="29.28515625" style="10" customWidth="1"/>
     <col min="23" max="23" width="53" style="10" customWidth="1"/>
-    <col min="24" max="16384" width="10.88671875" style="10"/>
+    <col min="24" max="16384" width="10.85546875" style="10"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="64" t="s">
+    <row r="1" spans="1:23" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="32" t="s">
         <v>32</v>
       </c>
-      <c r="B1" s="61" t="s">
+      <c r="B1" s="26" t="s">
         <v>54</v>
       </c>
-      <c r="C1" s="61" t="s">
+      <c r="C1" s="26" t="s">
         <v>53</v>
       </c>
-      <c r="D1" s="44" t="s">
+      <c r="D1" s="29" t="s">
         <v>50</v>
       </c>
-      <c r="E1" s="44" t="s">
+      <c r="E1" s="29" t="s">
         <v>48</v>
       </c>
-      <c r="F1" s="59" t="s">
+      <c r="F1" s="45" t="s">
         <v>55</v>
       </c>
-      <c r="G1" s="59"/>
-      <c r="H1" s="59"/>
-      <c r="I1" s="59"/>
-      <c r="J1" s="59"/>
-      <c r="K1" s="59"/>
-      <c r="L1" s="59"/>
-      <c r="M1" s="59"/>
-      <c r="N1" s="59"/>
-      <c r="O1" s="59"/>
-      <c r="P1" s="59"/>
-      <c r="Q1" s="59"/>
-      <c r="R1" s="59"/>
-      <c r="S1" s="59"/>
-      <c r="T1" s="60"/>
+      <c r="G1" s="45"/>
+      <c r="H1" s="45"/>
+      <c r="I1" s="45"/>
+      <c r="J1" s="45"/>
+      <c r="K1" s="45"/>
+      <c r="L1" s="45"/>
+      <c r="M1" s="45"/>
+      <c r="N1" s="45"/>
+      <c r="O1" s="45"/>
+      <c r="P1" s="45"/>
+      <c r="Q1" s="45"/>
+      <c r="R1" s="45"/>
+      <c r="S1" s="45"/>
+      <c r="T1" s="46"/>
       <c r="U1" s="16"/>
-      <c r="V1" s="44" t="s">
+      <c r="V1" s="29" t="s">
         <v>71</v>
       </c>
-      <c r="W1" s="44" t="s">
+      <c r="W1" s="29" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="2" spans="1:23" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="64"/>
-      <c r="B2" s="61"/>
-      <c r="C2" s="61"/>
-      <c r="D2" s="45"/>
-      <c r="E2" s="45"/>
-      <c r="F2" s="47" t="s">
+    <row r="2" spans="1:23" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="32"/>
+      <c r="B2" s="26"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="33" t="s">
         <v>95</v>
       </c>
-      <c r="G2" s="47"/>
-      <c r="H2" s="47"/>
-      <c r="I2" s="47"/>
-      <c r="J2" s="47"/>
-      <c r="K2" s="47"/>
-      <c r="L2" s="47"/>
-      <c r="M2" s="48"/>
-      <c r="N2" s="49" t="s">
+      <c r="G2" s="33"/>
+      <c r="H2" s="33"/>
+      <c r="I2" s="33"/>
+      <c r="J2" s="33"/>
+      <c r="K2" s="33"/>
+      <c r="L2" s="33"/>
+      <c r="M2" s="34"/>
+      <c r="N2" s="35" t="s">
         <v>44</v>
       </c>
-      <c r="O2" s="50"/>
-      <c r="P2" s="50"/>
-      <c r="Q2" s="50"/>
-      <c r="R2" s="50"/>
-      <c r="S2" s="50"/>
-      <c r="T2" s="51"/>
-      <c r="U2" s="55" t="s">
+      <c r="O2" s="36"/>
+      <c r="P2" s="36"/>
+      <c r="Q2" s="36"/>
+      <c r="R2" s="36"/>
+      <c r="S2" s="36"/>
+      <c r="T2" s="37"/>
+      <c r="U2" s="41" t="s">
         <v>67</v>
       </c>
-      <c r="V2" s="45"/>
-      <c r="W2" s="45"/>
-    </row>
-    <row r="3" spans="1:23" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="64"/>
-      <c r="B3" s="61"/>
-      <c r="C3" s="61"/>
-      <c r="D3" s="45"/>
-      <c r="E3" s="45"/>
-      <c r="F3" s="47" t="s">
+      <c r="V2" s="30"/>
+      <c r="W2" s="30"/>
+    </row>
+    <row r="3" spans="1:23" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="32"/>
+      <c r="B3" s="26"/>
+      <c r="C3" s="26"/>
+      <c r="D3" s="30"/>
+      <c r="E3" s="30"/>
+      <c r="F3" s="33" t="s">
         <v>45</v>
       </c>
-      <c r="G3" s="47"/>
-      <c r="H3" s="48"/>
-      <c r="I3" s="58" t="s">
+      <c r="G3" s="33"/>
+      <c r="H3" s="34"/>
+      <c r="I3" s="44" t="s">
         <v>47</v>
       </c>
-      <c r="J3" s="47"/>
-      <c r="K3" s="48"/>
-      <c r="L3" s="58" t="s">
+      <c r="J3" s="33"/>
+      <c r="K3" s="34"/>
+      <c r="L3" s="44" t="s">
         <v>46</v>
       </c>
-      <c r="M3" s="48"/>
-      <c r="N3" s="52"/>
-      <c r="O3" s="53"/>
-      <c r="P3" s="53"/>
-      <c r="Q3" s="53"/>
-      <c r="R3" s="53"/>
-      <c r="S3" s="53"/>
-      <c r="T3" s="54"/>
-      <c r="U3" s="56"/>
-      <c r="V3" s="45"/>
-      <c r="W3" s="45"/>
-    </row>
-    <row r="4" spans="1:23" ht="113.4" x14ac:dyDescent="0.25">
+      <c r="M3" s="34"/>
+      <c r="N3" s="38"/>
+      <c r="O3" s="39"/>
+      <c r="P3" s="39"/>
+      <c r="Q3" s="39"/>
+      <c r="R3" s="39"/>
+      <c r="S3" s="39"/>
+      <c r="T3" s="40"/>
+      <c r="U3" s="42"/>
+      <c r="V3" s="30"/>
+      <c r="W3" s="30"/>
+    </row>
+    <row r="4" spans="1:23" ht="114" x14ac:dyDescent="0.2">
       <c r="A4" s="15" t="s">
         <v>86</v>
       </c>
-      <c r="B4" s="61"/>
-      <c r="C4" s="61"/>
-      <c r="D4" s="46"/>
-      <c r="E4" s="46"/>
+      <c r="B4" s="26"/>
+      <c r="C4" s="26"/>
+      <c r="D4" s="31"/>
+      <c r="E4" s="31"/>
       <c r="F4" s="11" t="s">
         <v>57</v>
       </c>
@@ -3461,11 +3461,11 @@
       <c r="T4" s="11" t="s">
         <v>81</v>
       </c>
-      <c r="U4" s="57"/>
-      <c r="V4" s="46"/>
-      <c r="W4" s="46"/>
-    </row>
-    <row r="5" spans="1:23" ht="122.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="U4" s="43"/>
+      <c r="V4" s="31"/>
+      <c r="W4" s="31"/>
+    </row>
+    <row r="5" spans="1:23" ht="122.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="24"/>
       <c r="B5" s="9"/>
       <c r="C5" s="9"/>
@@ -3490,7 +3490,7 @@
       <c r="V5" s="9"/>
       <c r="W5" s="9"/>
     </row>
-    <row r="6" spans="1:23" ht="148.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:23" ht="148.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="24"/>
       <c r="B6" s="9"/>
       <c r="C6" s="9"/>
@@ -3515,7 +3515,7 @@
       <c r="V6" s="9"/>
       <c r="W6" s="9"/>
     </row>
-    <row r="7" spans="1:23" ht="132.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:23" ht="132.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="24"/>
       <c r="B7" s="9"/>
       <c r="C7" s="9"/>
@@ -3540,7 +3540,7 @@
       <c r="V7" s="9"/>
       <c r="W7" s="9"/>
     </row>
-    <row r="8" spans="1:23" ht="81" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:23" ht="81" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="24"/>
       <c r="B8" s="9"/>
       <c r="C8" s="9"/>
@@ -3565,7 +3565,7 @@
       <c r="V8" s="9"/>
       <c r="W8" s="9"/>
     </row>
-    <row r="9" spans="1:23" ht="129" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:23" ht="129" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="24"/>
       <c r="B9" s="9"/>
       <c r="C9" s="9"/>
@@ -3590,7 +3590,7 @@
       <c r="V9" s="9"/>
       <c r="W9" s="9"/>
     </row>
-    <row r="10" spans="1:23" ht="72.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:23" ht="72.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="25"/>
       <c r="B10" s="9"/>
       <c r="C10" s="9"/>
@@ -3615,7 +3615,7 @@
       <c r="V10" s="9"/>
       <c r="W10" s="9"/>
     </row>
-    <row r="11" spans="1:23" ht="89.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:23" ht="89.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="25"/>
       <c r="B11" s="9"/>
       <c r="C11" s="9"/>
@@ -3640,7 +3640,7 @@
       <c r="V11" s="9"/>
       <c r="W11" s="9"/>
     </row>
-    <row r="12" spans="1:23" ht="108.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:23" ht="108.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="25"/>
       <c r="B12" s="9"/>
       <c r="C12" s="9"/>
@@ -3665,7 +3665,7 @@
       <c r="V12" s="9"/>
       <c r="W12" s="9"/>
     </row>
-    <row r="13" spans="1:23" ht="85.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:23" ht="85.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="25"/>
       <c r="B13" s="9"/>
       <c r="C13" s="9"/>
@@ -3690,7 +3690,7 @@
       <c r="V13" s="12"/>
       <c r="W13" s="12"/>
     </row>
-    <row r="14" spans="1:23" ht="83.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:23" ht="83.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="25"/>
       <c r="B14" s="9"/>
       <c r="C14" s="9"/>
@@ -3715,7 +3715,7 @@
       <c r="V14" s="12"/>
       <c r="W14" s="12"/>
     </row>
-    <row r="15" spans="1:23" ht="81" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:23" ht="81" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="25"/>
       <c r="B15" s="9"/>
       <c r="C15" s="9"/>
@@ -3740,41 +3740,50 @@
       <c r="V15" s="12"/>
       <c r="W15" s="12"/>
     </row>
-    <row r="24" spans="1:5" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="62" t="s">
+    <row r="24" spans="1:5" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A24" s="27" t="s">
         <v>94</v>
       </c>
-      <c r="B24" s="62"/>
-      <c r="C24" s="62"/>
-      <c r="D24" s="62"/>
-      <c r="E24" s="63"/>
-    </row>
-    <row r="25" spans="1:5" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="62"/>
-      <c r="B25" s="62"/>
-      <c r="C25" s="62"/>
-      <c r="D25" s="62"/>
-      <c r="E25" s="63"/>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A26" s="62" t="s">
+      <c r="B24" s="27"/>
+      <c r="C24" s="27"/>
+      <c r="D24" s="27"/>
+      <c r="E24" s="28"/>
+    </row>
+    <row r="25" spans="1:5" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A25" s="27"/>
+      <c r="B25" s="27"/>
+      <c r="C25" s="27"/>
+      <c r="D25" s="27"/>
+      <c r="E25" s="28"/>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A26" s="27" t="s">
         <v>91</v>
       </c>
-      <c r="B26" s="62"/>
-      <c r="C26" s="62"/>
-      <c r="D26" s="62"/>
-      <c r="E26" s="63"/>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A27" s="62"/>
-      <c r="B27" s="62"/>
-      <c r="C27" s="62"/>
-      <c r="D27" s="62"/>
-      <c r="E27" s="63"/>
+      <c r="B26" s="27"/>
+      <c r="C26" s="27"/>
+      <c r="D26" s="27"/>
+      <c r="E26" s="28"/>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A27" s="27"/>
+      <c r="B27" s="27"/>
+      <c r="C27" s="27"/>
+      <c r="D27" s="27"/>
+      <c r="E27" s="28"/>
     </row>
   </sheetData>
   <dataConsolidate/>
   <mergeCells count="18">
+    <mergeCell ref="W1:W4"/>
+    <mergeCell ref="F2:M2"/>
+    <mergeCell ref="N2:T3"/>
+    <mergeCell ref="U2:U4"/>
+    <mergeCell ref="F3:H3"/>
+    <mergeCell ref="I3:K3"/>
+    <mergeCell ref="L3:M3"/>
+    <mergeCell ref="V1:V4"/>
+    <mergeCell ref="F1:T1"/>
     <mergeCell ref="B1:B4"/>
     <mergeCell ref="A24:D25"/>
     <mergeCell ref="E24:E25"/>
@@ -3784,15 +3793,6 @@
     <mergeCell ref="D1:D4"/>
     <mergeCell ref="E1:E4"/>
     <mergeCell ref="A1:A3"/>
-    <mergeCell ref="W1:W4"/>
-    <mergeCell ref="F2:M2"/>
-    <mergeCell ref="N2:T3"/>
-    <mergeCell ref="U2:U4"/>
-    <mergeCell ref="F3:H3"/>
-    <mergeCell ref="I3:K3"/>
-    <mergeCell ref="L3:M3"/>
-    <mergeCell ref="V1:V4"/>
-    <mergeCell ref="F1:T1"/>
   </mergeCells>
   <conditionalFormatting sqref="T5:T15">
     <cfRule type="containsText" dxfId="3" priority="1" stopIfTrue="1" operator="containsText" text="SI">
@@ -3851,140 +3851,140 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A2:X29"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.88671875" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="31.88671875" style="10" customWidth="1"/>
+    <col min="1" max="1" width="31.85546875" style="10" customWidth="1"/>
     <col min="2" max="3" width="7" style="10" customWidth="1"/>
-    <col min="4" max="4" width="39.33203125" style="10" customWidth="1"/>
+    <col min="4" max="4" width="39.28515625" style="10" customWidth="1"/>
     <col min="5" max="5" width="21" style="10" customWidth="1"/>
-    <col min="6" max="7" width="5.88671875" style="10" customWidth="1"/>
-    <col min="8" max="8" width="6.33203125" style="10" customWidth="1"/>
+    <col min="6" max="7" width="5.85546875" style="10" customWidth="1"/>
+    <col min="8" max="8" width="6.28515625" style="10" customWidth="1"/>
     <col min="9" max="9" width="6" style="10" customWidth="1"/>
-    <col min="10" max="10" width="6.44140625" style="10" customWidth="1"/>
-    <col min="11" max="18" width="5.44140625" style="10" customWidth="1"/>
-    <col min="19" max="19" width="4.33203125" style="10" customWidth="1"/>
+    <col min="10" max="10" width="6.42578125" style="10" customWidth="1"/>
+    <col min="11" max="18" width="5.42578125" style="10" customWidth="1"/>
+    <col min="19" max="19" width="4.28515625" style="10" customWidth="1"/>
     <col min="20" max="20" width="3" style="10" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="6.44140625" style="10" customWidth="1"/>
+    <col min="21" max="21" width="6.42578125" style="10" customWidth="1"/>
     <col min="22" max="22" width="11" style="10" customWidth="1"/>
-    <col min="23" max="23" width="29.33203125" style="10" customWidth="1"/>
-    <col min="24" max="24" width="42.5546875" style="10" customWidth="1"/>
-    <col min="25" max="16384" width="10.88671875" style="10"/>
+    <col min="23" max="23" width="29.28515625" style="10" customWidth="1"/>
+    <col min="24" max="24" width="42.5703125" style="10" customWidth="1"/>
+    <col min="25" max="16384" width="10.85546875" style="10"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:24" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="68" t="s">
+    <row r="2" spans="1:24" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="67" t="s">
         <v>32</v>
       </c>
-      <c r="B2" s="61" t="s">
+      <c r="B2" s="26" t="s">
         <v>54</v>
       </c>
-      <c r="C2" s="66" t="s">
+      <c r="C2" s="65" t="s">
         <v>53</v>
       </c>
-      <c r="D2" s="44" t="s">
+      <c r="D2" s="29" t="s">
         <v>50</v>
       </c>
-      <c r="E2" s="44" t="s">
+      <c r="E2" s="29" t="s">
         <v>48</v>
       </c>
-      <c r="F2" s="65" t="s">
+      <c r="F2" s="69" t="s">
         <v>55</v>
       </c>
-      <c r="G2" s="59"/>
-      <c r="H2" s="59"/>
-      <c r="I2" s="59"/>
-      <c r="J2" s="59"/>
-      <c r="K2" s="59"/>
-      <c r="L2" s="59"/>
-      <c r="M2" s="59"/>
-      <c r="N2" s="59"/>
-      <c r="O2" s="59"/>
-      <c r="P2" s="59"/>
-      <c r="Q2" s="59"/>
-      <c r="R2" s="59"/>
-      <c r="S2" s="59"/>
-      <c r="T2" s="59"/>
-      <c r="U2" s="60"/>
+      <c r="G2" s="45"/>
+      <c r="H2" s="45"/>
+      <c r="I2" s="45"/>
+      <c r="J2" s="45"/>
+      <c r="K2" s="45"/>
+      <c r="L2" s="45"/>
+      <c r="M2" s="45"/>
+      <c r="N2" s="45"/>
+      <c r="O2" s="45"/>
+      <c r="P2" s="45"/>
+      <c r="Q2" s="45"/>
+      <c r="R2" s="45"/>
+      <c r="S2" s="45"/>
+      <c r="T2" s="45"/>
+      <c r="U2" s="46"/>
       <c r="V2" s="16"/>
-      <c r="W2" s="44" t="s">
+      <c r="W2" s="29" t="s">
         <v>71</v>
       </c>
-      <c r="X2" s="44" t="s">
+      <c r="X2" s="29" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="3" spans="1:24" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="68"/>
-      <c r="B3" s="61"/>
-      <c r="C3" s="66"/>
-      <c r="D3" s="45"/>
-      <c r="E3" s="45"/>
-      <c r="F3" s="58" t="s">
+    <row r="3" spans="1:24" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="67"/>
+      <c r="B3" s="26"/>
+      <c r="C3" s="65"/>
+      <c r="D3" s="30"/>
+      <c r="E3" s="30"/>
+      <c r="F3" s="44" t="s">
         <v>49</v>
       </c>
-      <c r="G3" s="47"/>
-      <c r="H3" s="47"/>
-      <c r="I3" s="47"/>
-      <c r="J3" s="47"/>
-      <c r="K3" s="47"/>
-      <c r="L3" s="47"/>
-      <c r="M3" s="47"/>
-      <c r="N3" s="48"/>
-      <c r="O3" s="49" t="s">
+      <c r="G3" s="33"/>
+      <c r="H3" s="33"/>
+      <c r="I3" s="33"/>
+      <c r="J3" s="33"/>
+      <c r="K3" s="33"/>
+      <c r="L3" s="33"/>
+      <c r="M3" s="33"/>
+      <c r="N3" s="34"/>
+      <c r="O3" s="35" t="s">
         <v>44</v>
       </c>
-      <c r="P3" s="50"/>
-      <c r="Q3" s="50"/>
-      <c r="R3" s="50"/>
-      <c r="S3" s="50"/>
-      <c r="T3" s="50"/>
-      <c r="U3" s="51"/>
-      <c r="V3" s="55" t="s">
+      <c r="P3" s="36"/>
+      <c r="Q3" s="36"/>
+      <c r="R3" s="36"/>
+      <c r="S3" s="36"/>
+      <c r="T3" s="36"/>
+      <c r="U3" s="37"/>
+      <c r="V3" s="41" t="s">
         <v>67</v>
       </c>
-      <c r="W3" s="45"/>
-      <c r="X3" s="45"/>
-    </row>
-    <row r="4" spans="1:24" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="69"/>
-      <c r="B4" s="61"/>
-      <c r="C4" s="66"/>
-      <c r="D4" s="45"/>
-      <c r="E4" s="45"/>
-      <c r="F4" s="58" t="s">
+      <c r="W3" s="30"/>
+      <c r="X3" s="30"/>
+    </row>
+    <row r="4" spans="1:24" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="68"/>
+      <c r="B4" s="26"/>
+      <c r="C4" s="65"/>
+      <c r="D4" s="30"/>
+      <c r="E4" s="30"/>
+      <c r="F4" s="44" t="s">
         <v>45</v>
       </c>
-      <c r="G4" s="47"/>
-      <c r="H4" s="47"/>
-      <c r="I4" s="48"/>
-      <c r="J4" s="58" t="s">
+      <c r="G4" s="33"/>
+      <c r="H4" s="33"/>
+      <c r="I4" s="34"/>
+      <c r="J4" s="44" t="s">
         <v>47</v>
       </c>
-      <c r="K4" s="47"/>
-      <c r="L4" s="48"/>
-      <c r="M4" s="58" t="s">
+      <c r="K4" s="33"/>
+      <c r="L4" s="34"/>
+      <c r="M4" s="44" t="s">
         <v>46</v>
       </c>
-      <c r="N4" s="48"/>
-      <c r="O4" s="52"/>
-      <c r="P4" s="53"/>
-      <c r="Q4" s="53"/>
-      <c r="R4" s="53"/>
-      <c r="S4" s="53"/>
-      <c r="T4" s="53"/>
-      <c r="U4" s="54"/>
-      <c r="V4" s="56"/>
-      <c r="W4" s="45"/>
-      <c r="X4" s="45"/>
-    </row>
-    <row r="5" spans="1:24" ht="113.4" x14ac:dyDescent="0.25">
+      <c r="N4" s="34"/>
+      <c r="O4" s="38"/>
+      <c r="P4" s="39"/>
+      <c r="Q4" s="39"/>
+      <c r="R4" s="39"/>
+      <c r="S4" s="39"/>
+      <c r="T4" s="39"/>
+      <c r="U4" s="40"/>
+      <c r="V4" s="42"/>
+      <c r="W4" s="30"/>
+      <c r="X4" s="30"/>
+    </row>
+    <row r="5" spans="1:24" ht="114" x14ac:dyDescent="0.2">
       <c r="A5" s="15" t="s">
         <v>87</v>
       </c>
-      <c r="B5" s="61"/>
-      <c r="C5" s="67"/>
-      <c r="D5" s="46"/>
-      <c r="E5" s="46"/>
+      <c r="B5" s="26"/>
+      <c r="C5" s="66"/>
+      <c r="D5" s="31"/>
+      <c r="E5" s="31"/>
       <c r="F5" s="11" t="s">
         <v>56</v>
       </c>
@@ -4033,11 +4033,11 @@
       <c r="U5" s="11" t="s">
         <v>81</v>
       </c>
-      <c r="V5" s="57"/>
-      <c r="W5" s="46"/>
-      <c r="X5" s="46"/>
-    </row>
-    <row r="6" spans="1:24" ht="87.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="V5" s="43"/>
+      <c r="W5" s="31"/>
+      <c r="X5" s="31"/>
+    </row>
+    <row r="6" spans="1:24" ht="87.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="24"/>
       <c r="B6" s="9"/>
       <c r="C6" s="9"/>
@@ -4063,7 +4063,7 @@
       <c r="W6" s="9"/>
       <c r="X6" s="9"/>
     </row>
-    <row r="7" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A7" s="24"/>
       <c r="B7" s="9"/>
       <c r="C7" s="9"/>
@@ -4089,7 +4089,7 @@
       <c r="W7" s="9"/>
       <c r="X7" s="9"/>
     </row>
-    <row r="8" spans="1:24" ht="108.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:24" ht="108.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="24"/>
       <c r="B8" s="9"/>
       <c r="C8" s="9"/>
@@ -4115,7 +4115,7 @@
       <c r="W8" s="9"/>
       <c r="X8" s="9"/>
     </row>
-    <row r="9" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A9" s="25"/>
       <c r="B9" s="9"/>
       <c r="C9" s="9"/>
@@ -4141,7 +4141,7 @@
       <c r="W9" s="9"/>
       <c r="X9" s="9"/>
     </row>
-    <row r="10" spans="1:24" ht="68.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:24" ht="68.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="25"/>
       <c r="B10" s="9"/>
       <c r="C10" s="9"/>
@@ -4167,7 +4167,7 @@
       <c r="W10" s="9"/>
       <c r="X10" s="9"/>
     </row>
-    <row r="11" spans="1:24" ht="89.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:24" ht="89.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="25"/>
       <c r="B11" s="9"/>
       <c r="C11" s="9"/>
@@ -4193,7 +4193,7 @@
       <c r="W11" s="9"/>
       <c r="X11" s="9"/>
     </row>
-    <row r="12" spans="1:24" ht="144" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:24" ht="144" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="25"/>
       <c r="B12" s="9"/>
       <c r="C12" s="9"/>
@@ -4219,7 +4219,7 @@
       <c r="W12" s="9"/>
       <c r="X12" s="9"/>
     </row>
-    <row r="13" spans="1:24" ht="80.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:24" ht="80.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="25"/>
       <c r="B13" s="9"/>
       <c r="C13" s="9"/>
@@ -4245,7 +4245,7 @@
       <c r="W13" s="12"/>
       <c r="X13" s="12"/>
     </row>
-    <row r="14" spans="1:24" ht="99" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:24" ht="99" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="25"/>
       <c r="B14" s="9"/>
       <c r="C14" s="9"/>
@@ -4271,41 +4271,50 @@
       <c r="W14" s="12"/>
       <c r="X14" s="12"/>
     </row>
-    <row r="26" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="62" t="s">
+    <row r="26" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A26" s="27" t="s">
         <v>92</v>
       </c>
-      <c r="B26" s="62"/>
-      <c r="C26" s="62"/>
-      <c r="D26" s="62"/>
-      <c r="E26" s="63"/>
-    </row>
-    <row r="27" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="62"/>
-      <c r="B27" s="62"/>
-      <c r="C27" s="62"/>
-      <c r="D27" s="62"/>
-      <c r="E27" s="63"/>
-    </row>
-    <row r="28" spans="1:5" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="62" t="s">
+      <c r="B26" s="27"/>
+      <c r="C26" s="27"/>
+      <c r="D26" s="27"/>
+      <c r="E26" s="28"/>
+    </row>
+    <row r="27" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A27" s="27"/>
+      <c r="B27" s="27"/>
+      <c r="C27" s="27"/>
+      <c r="D27" s="27"/>
+      <c r="E27" s="28"/>
+    </row>
+    <row r="28" spans="1:5" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A28" s="27" t="s">
         <v>91</v>
       </c>
-      <c r="B28" s="62"/>
-      <c r="C28" s="62"/>
-      <c r="D28" s="62"/>
-      <c r="E28" s="63"/>
-    </row>
-    <row r="29" spans="1:5" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="62"/>
-      <c r="B29" s="62"/>
-      <c r="C29" s="62"/>
-      <c r="D29" s="62"/>
-      <c r="E29" s="63"/>
+      <c r="B28" s="27"/>
+      <c r="C28" s="27"/>
+      <c r="D28" s="27"/>
+      <c r="E28" s="28"/>
+    </row>
+    <row r="29" spans="1:5" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A29" s="27"/>
+      <c r="B29" s="27"/>
+      <c r="C29" s="27"/>
+      <c r="D29" s="27"/>
+      <c r="E29" s="28"/>
     </row>
   </sheetData>
   <dataConsolidate/>
   <mergeCells count="18">
+    <mergeCell ref="X2:X5"/>
+    <mergeCell ref="F3:N3"/>
+    <mergeCell ref="O3:U4"/>
+    <mergeCell ref="V3:V5"/>
+    <mergeCell ref="F4:I4"/>
+    <mergeCell ref="J4:L4"/>
+    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="W2:W5"/>
+    <mergeCell ref="F2:U2"/>
     <mergeCell ref="B2:B5"/>
     <mergeCell ref="A26:D27"/>
     <mergeCell ref="A28:D29"/>
@@ -4315,15 +4324,6 @@
     <mergeCell ref="E2:E5"/>
     <mergeCell ref="A2:A4"/>
     <mergeCell ref="E26:E27"/>
-    <mergeCell ref="X2:X5"/>
-    <mergeCell ref="F3:N3"/>
-    <mergeCell ref="O3:U4"/>
-    <mergeCell ref="V3:V5"/>
-    <mergeCell ref="F4:I4"/>
-    <mergeCell ref="J4:L4"/>
-    <mergeCell ref="M4:N4"/>
-    <mergeCell ref="W2:W5"/>
-    <mergeCell ref="F2:U2"/>
   </mergeCells>
   <conditionalFormatting sqref="U6:U14">
     <cfRule type="containsText" dxfId="2" priority="18" stopIfTrue="1" operator="containsText" text="SI">
@@ -4382,140 +4382,140 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A2:X32"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.88671875" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="31.88671875" style="10" customWidth="1"/>
-    <col min="2" max="2" width="11.5546875" style="10" customWidth="1"/>
-    <col min="3" max="3" width="6.44140625" style="10" customWidth="1"/>
-    <col min="4" max="4" width="33.6640625" style="10" customWidth="1"/>
+    <col min="1" max="1" width="31.85546875" style="10" customWidth="1"/>
+    <col min="2" max="2" width="11.5703125" style="10" customWidth="1"/>
+    <col min="3" max="3" width="6.42578125" style="10" customWidth="1"/>
+    <col min="4" max="4" width="33.7109375" style="10" customWidth="1"/>
     <col min="5" max="5" width="21" style="10" customWidth="1"/>
-    <col min="6" max="7" width="5.88671875" style="10" customWidth="1"/>
-    <col min="8" max="8" width="6.33203125" style="10" customWidth="1"/>
+    <col min="6" max="7" width="5.85546875" style="10" customWidth="1"/>
+    <col min="8" max="8" width="6.28515625" style="10" customWidth="1"/>
     <col min="9" max="9" width="6" style="10" customWidth="1"/>
-    <col min="10" max="10" width="6.44140625" style="10" customWidth="1"/>
-    <col min="11" max="18" width="5.44140625" style="10" customWidth="1"/>
-    <col min="19" max="19" width="4.33203125" style="10" customWidth="1"/>
+    <col min="10" max="10" width="6.42578125" style="10" customWidth="1"/>
+    <col min="11" max="18" width="5.42578125" style="10" customWidth="1"/>
+    <col min="19" max="19" width="4.28515625" style="10" customWidth="1"/>
     <col min="20" max="20" width="3" style="10" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="6.44140625" style="10" customWidth="1"/>
+    <col min="21" max="21" width="6.42578125" style="10" customWidth="1"/>
     <col min="22" max="22" width="11" style="10" customWidth="1"/>
-    <col min="23" max="24" width="29.33203125" style="10" customWidth="1"/>
-    <col min="25" max="16384" width="10.88671875" style="10"/>
+    <col min="23" max="24" width="29.28515625" style="10" customWidth="1"/>
+    <col min="25" max="16384" width="10.85546875" style="10"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:24" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="68" t="s">
+    <row r="2" spans="1:24" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="67" t="s">
         <v>32</v>
       </c>
-      <c r="B2" s="61" t="s">
+      <c r="B2" s="26" t="s">
         <v>54</v>
       </c>
-      <c r="C2" s="66" t="s">
+      <c r="C2" s="65" t="s">
         <v>53</v>
       </c>
-      <c r="D2" s="44" t="s">
+      <c r="D2" s="29" t="s">
         <v>50</v>
       </c>
-      <c r="E2" s="44" t="s">
+      <c r="E2" s="29" t="s">
         <v>48</v>
       </c>
-      <c r="F2" s="65" t="s">
+      <c r="F2" s="69" t="s">
         <v>55</v>
       </c>
-      <c r="G2" s="59"/>
-      <c r="H2" s="59"/>
-      <c r="I2" s="59"/>
-      <c r="J2" s="59"/>
-      <c r="K2" s="59"/>
-      <c r="L2" s="59"/>
-      <c r="M2" s="59"/>
-      <c r="N2" s="59"/>
-      <c r="O2" s="59"/>
-      <c r="P2" s="59"/>
-      <c r="Q2" s="59"/>
-      <c r="R2" s="59"/>
-      <c r="S2" s="59"/>
-      <c r="T2" s="59"/>
-      <c r="U2" s="60"/>
+      <c r="G2" s="45"/>
+      <c r="H2" s="45"/>
+      <c r="I2" s="45"/>
+      <c r="J2" s="45"/>
+      <c r="K2" s="45"/>
+      <c r="L2" s="45"/>
+      <c r="M2" s="45"/>
+      <c r="N2" s="45"/>
+      <c r="O2" s="45"/>
+      <c r="P2" s="45"/>
+      <c r="Q2" s="45"/>
+      <c r="R2" s="45"/>
+      <c r="S2" s="45"/>
+      <c r="T2" s="45"/>
+      <c r="U2" s="46"/>
       <c r="V2" s="16"/>
-      <c r="W2" s="44" t="s">
+      <c r="W2" s="29" t="s">
         <v>71</v>
       </c>
-      <c r="X2" s="44" t="s">
+      <c r="X2" s="29" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="3" spans="1:24" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="68"/>
-      <c r="B3" s="61"/>
-      <c r="C3" s="66"/>
-      <c r="D3" s="45"/>
-      <c r="E3" s="45"/>
-      <c r="F3" s="58" t="s">
+    <row r="3" spans="1:24" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="67"/>
+      <c r="B3" s="26"/>
+      <c r="C3" s="65"/>
+      <c r="D3" s="30"/>
+      <c r="E3" s="30"/>
+      <c r="F3" s="44" t="s">
         <v>49</v>
       </c>
-      <c r="G3" s="47"/>
-      <c r="H3" s="47"/>
-      <c r="I3" s="47"/>
-      <c r="J3" s="47"/>
-      <c r="K3" s="47"/>
-      <c r="L3" s="47"/>
-      <c r="M3" s="47"/>
-      <c r="N3" s="48"/>
-      <c r="O3" s="49" t="s">
+      <c r="G3" s="33"/>
+      <c r="H3" s="33"/>
+      <c r="I3" s="33"/>
+      <c r="J3" s="33"/>
+      <c r="K3" s="33"/>
+      <c r="L3" s="33"/>
+      <c r="M3" s="33"/>
+      <c r="N3" s="34"/>
+      <c r="O3" s="35" t="s">
         <v>44</v>
       </c>
-      <c r="P3" s="50"/>
-      <c r="Q3" s="50"/>
-      <c r="R3" s="50"/>
-      <c r="S3" s="50"/>
-      <c r="T3" s="50"/>
-      <c r="U3" s="51"/>
-      <c r="V3" s="55" t="s">
+      <c r="P3" s="36"/>
+      <c r="Q3" s="36"/>
+      <c r="R3" s="36"/>
+      <c r="S3" s="36"/>
+      <c r="T3" s="36"/>
+      <c r="U3" s="37"/>
+      <c r="V3" s="41" t="s">
         <v>67</v>
       </c>
-      <c r="W3" s="45"/>
-      <c r="X3" s="45"/>
-    </row>
-    <row r="4" spans="1:24" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="69"/>
-      <c r="B4" s="61"/>
-      <c r="C4" s="66"/>
-      <c r="D4" s="45"/>
-      <c r="E4" s="45"/>
-      <c r="F4" s="58" t="s">
+      <c r="W3" s="30"/>
+      <c r="X3" s="30"/>
+    </row>
+    <row r="4" spans="1:24" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="68"/>
+      <c r="B4" s="26"/>
+      <c r="C4" s="65"/>
+      <c r="D4" s="30"/>
+      <c r="E4" s="30"/>
+      <c r="F4" s="44" t="s">
         <v>45</v>
       </c>
-      <c r="G4" s="47"/>
-      <c r="H4" s="47"/>
-      <c r="I4" s="48"/>
-      <c r="J4" s="58" t="s">
+      <c r="G4" s="33"/>
+      <c r="H4" s="33"/>
+      <c r="I4" s="34"/>
+      <c r="J4" s="44" t="s">
         <v>47</v>
       </c>
-      <c r="K4" s="47"/>
-      <c r="L4" s="48"/>
-      <c r="M4" s="58" t="s">
+      <c r="K4" s="33"/>
+      <c r="L4" s="34"/>
+      <c r="M4" s="44" t="s">
         <v>46</v>
       </c>
-      <c r="N4" s="48"/>
-      <c r="O4" s="52"/>
-      <c r="P4" s="53"/>
-      <c r="Q4" s="53"/>
-      <c r="R4" s="53"/>
-      <c r="S4" s="53"/>
-      <c r="T4" s="53"/>
-      <c r="U4" s="54"/>
-      <c r="V4" s="56"/>
-      <c r="W4" s="45"/>
-      <c r="X4" s="45"/>
-    </row>
-    <row r="5" spans="1:24" ht="113.4" x14ac:dyDescent="0.25">
+      <c r="N4" s="34"/>
+      <c r="O4" s="38"/>
+      <c r="P4" s="39"/>
+      <c r="Q4" s="39"/>
+      <c r="R4" s="39"/>
+      <c r="S4" s="39"/>
+      <c r="T4" s="39"/>
+      <c r="U4" s="40"/>
+      <c r="V4" s="42"/>
+      <c r="W4" s="30"/>
+      <c r="X4" s="30"/>
+    </row>
+    <row r="5" spans="1:24" ht="114" x14ac:dyDescent="0.2">
       <c r="A5" s="15" t="s">
         <v>88</v>
       </c>
-      <c r="B5" s="61"/>
-      <c r="C5" s="67"/>
-      <c r="D5" s="46"/>
-      <c r="E5" s="46"/>
+      <c r="B5" s="26"/>
+      <c r="C5" s="66"/>
+      <c r="D5" s="31"/>
+      <c r="E5" s="31"/>
       <c r="F5" s="11" t="s">
         <v>56</v>
       </c>
@@ -4564,11 +4564,11 @@
       <c r="U5" s="11" t="s">
         <v>81</v>
       </c>
-      <c r="V5" s="57"/>
-      <c r="W5" s="46"/>
-      <c r="X5" s="46"/>
-    </row>
-    <row r="6" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="V5" s="43"/>
+      <c r="W5" s="31"/>
+      <c r="X5" s="31"/>
+    </row>
+    <row r="6" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A6" s="70"/>
       <c r="B6" s="9"/>
       <c r="C6" s="9"/>
@@ -4594,7 +4594,7 @@
       <c r="W6" s="9"/>
       <c r="X6" s="9"/>
     </row>
-    <row r="7" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A7" s="71"/>
       <c r="B7" s="9"/>
       <c r="C7" s="9"/>
@@ -4620,7 +4620,7 @@
       <c r="W7" s="9"/>
       <c r="X7" s="9"/>
     </row>
-    <row r="8" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A8" s="71"/>
       <c r="B8" s="9"/>
       <c r="C8" s="9"/>
@@ -4646,7 +4646,7 @@
       <c r="W8" s="9"/>
       <c r="X8" s="9"/>
     </row>
-    <row r="9" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A9" s="71"/>
       <c r="B9" s="9"/>
       <c r="C9" s="9"/>
@@ -4672,7 +4672,7 @@
       <c r="W9" s="9"/>
       <c r="X9" s="9"/>
     </row>
-    <row r="10" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A10" s="71"/>
       <c r="B10" s="9"/>
       <c r="C10" s="9"/>
@@ -4698,7 +4698,7 @@
       <c r="W10" s="9"/>
       <c r="X10" s="9"/>
     </row>
-    <row r="11" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A11" s="71"/>
       <c r="B11" s="9"/>
       <c r="C11" s="9"/>
@@ -4724,7 +4724,7 @@
       <c r="W11" s="9"/>
       <c r="X11" s="9"/>
     </row>
-    <row r="12" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A12" s="71"/>
       <c r="B12" s="9"/>
       <c r="C12" s="9"/>
@@ -4750,7 +4750,7 @@
       <c r="W12" s="9"/>
       <c r="X12" s="9"/>
     </row>
-    <row r="13" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A13" s="71"/>
       <c r="B13" s="9"/>
       <c r="C13" s="9"/>
@@ -4776,7 +4776,7 @@
       <c r="W13" s="9"/>
       <c r="X13" s="9"/>
     </row>
-    <row r="14" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A14" s="71"/>
       <c r="B14" s="9"/>
       <c r="C14" s="9"/>
@@ -4802,7 +4802,7 @@
       <c r="W14" s="9"/>
       <c r="X14" s="9"/>
     </row>
-    <row r="15" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A15" s="71"/>
       <c r="B15" s="9"/>
       <c r="C15" s="9"/>
@@ -4828,7 +4828,7 @@
       <c r="W15" s="9"/>
       <c r="X15" s="9"/>
     </row>
-    <row r="16" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A16" s="71"/>
       <c r="B16" s="9"/>
       <c r="C16" s="9"/>
@@ -4854,7 +4854,7 @@
       <c r="W16" s="12"/>
       <c r="X16" s="12"/>
     </row>
-    <row r="17" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A17" s="71"/>
       <c r="B17" s="9"/>
       <c r="C17" s="9"/>
@@ -4880,7 +4880,7 @@
       <c r="W17" s="12"/>
       <c r="X17" s="12"/>
     </row>
-    <row r="18" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A18" s="72"/>
       <c r="B18" s="9"/>
       <c r="C18" s="9"/>
@@ -4906,41 +4906,50 @@
       <c r="W18" s="12"/>
       <c r="X18" s="12"/>
     </row>
-    <row r="29" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A29" s="62" t="s">
+    <row r="29" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A29" s="27" t="s">
         <v>92</v>
       </c>
-      <c r="B29" s="62"/>
-      <c r="C29" s="62"/>
-      <c r="D29" s="62"/>
-      <c r="E29" s="63"/>
-    </row>
-    <row r="30" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A30" s="62"/>
-      <c r="B30" s="62"/>
-      <c r="C30" s="62"/>
-      <c r="D30" s="62"/>
-      <c r="E30" s="63"/>
-    </row>
-    <row r="31" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A31" s="62" t="s">
+      <c r="B29" s="27"/>
+      <c r="C29" s="27"/>
+      <c r="D29" s="27"/>
+      <c r="E29" s="28"/>
+    </row>
+    <row r="30" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A30" s="27"/>
+      <c r="B30" s="27"/>
+      <c r="C30" s="27"/>
+      <c r="D30" s="27"/>
+      <c r="E30" s="28"/>
+    </row>
+    <row r="31" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A31" s="27" t="s">
         <v>91</v>
       </c>
-      <c r="B31" s="62"/>
-      <c r="C31" s="62"/>
-      <c r="D31" s="62"/>
-      <c r="E31" s="63"/>
-    </row>
-    <row r="32" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A32" s="62"/>
-      <c r="B32" s="62"/>
-      <c r="C32" s="62"/>
-      <c r="D32" s="62"/>
-      <c r="E32" s="63"/>
+      <c r="B31" s="27"/>
+      <c r="C31" s="27"/>
+      <c r="D31" s="27"/>
+      <c r="E31" s="28"/>
+    </row>
+    <row r="32" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A32" s="27"/>
+      <c r="B32" s="27"/>
+      <c r="C32" s="27"/>
+      <c r="D32" s="27"/>
+      <c r="E32" s="28"/>
     </row>
   </sheetData>
   <dataConsolidate/>
   <mergeCells count="19">
+    <mergeCell ref="X2:X5"/>
+    <mergeCell ref="F3:N3"/>
+    <mergeCell ref="O3:U4"/>
+    <mergeCell ref="V3:V5"/>
+    <mergeCell ref="F4:I4"/>
+    <mergeCell ref="J4:L4"/>
+    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="W2:W5"/>
+    <mergeCell ref="F2:U2"/>
     <mergeCell ref="B2:B5"/>
     <mergeCell ref="A29:D30"/>
     <mergeCell ref="E29:E30"/>
@@ -4951,15 +4960,6 @@
     <mergeCell ref="E2:E5"/>
     <mergeCell ref="A6:A18"/>
     <mergeCell ref="A2:A4"/>
-    <mergeCell ref="X2:X5"/>
-    <mergeCell ref="F3:N3"/>
-    <mergeCell ref="O3:U4"/>
-    <mergeCell ref="V3:V5"/>
-    <mergeCell ref="F4:I4"/>
-    <mergeCell ref="J4:L4"/>
-    <mergeCell ref="M4:N4"/>
-    <mergeCell ref="W2:W5"/>
-    <mergeCell ref="F2:U2"/>
   </mergeCells>
   <conditionalFormatting sqref="U6:U18">
     <cfRule type="containsText" dxfId="1" priority="1" stopIfTrue="1" operator="containsText" text="SI">
@@ -4979,10 +4979,10 @@
   <pageMargins left="0.70866141732283472" right="0.59055118110236227" top="1.1578124999999999" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="119" scale="47" fitToHeight="0" orientation="landscape" r:id="rId1"/>
   <headerFooter>
-    <oddHeader>&amp;C&amp;"Arial,Negrita"&amp;14&amp;KFF0000SUPERSERVICIO CUATRO CAMINOS S.A DE C.V&amp;K01+000
+    <oddHeader>&amp;C&amp;"Arial,Regular"&amp;14&amp;KFF0000SUPERSERVICIO CUATRO CAMINOS S.A DE C.V&amp;K01+000
 &amp;7TÍTULO
 &amp;11MATRIZ DE ASPECTOS E IMPACTOS AMBIENTALES
-&amp;"Arial,Normal"&amp;8Revisión Número: 0&amp;R&amp;9CLAVE: F-02-02           
+&amp;8Revisión Número: 0&amp;R&amp;9CLAVE: F-02-02           
    &amp;11    FECHA DE EMISIÓN:&amp;KFF000001/03/2019</oddHeader>
     <oddFooter>&amp;R&amp;P DE &amp;N</oddFooter>
   </headerFooter>
@@ -4990,7 +4990,7 @@
   <legacyDrawing r:id="rId3"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" disablePrompts="1" count="2">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0300-000000000000}">
           <x14:formula1>
             <xm:f>'Lista de AA'!$D$3:$D$18</xm:f>
@@ -5015,140 +5015,140 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A2:X32"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.88671875" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="31.88671875" style="10" customWidth="1"/>
-    <col min="2" max="2" width="11.5546875" style="10" customWidth="1"/>
-    <col min="3" max="3" width="6.44140625" style="10" customWidth="1"/>
-    <col min="4" max="4" width="35.6640625" style="10" customWidth="1"/>
+    <col min="1" max="1" width="31.85546875" style="10" customWidth="1"/>
+    <col min="2" max="2" width="11.5703125" style="10" customWidth="1"/>
+    <col min="3" max="3" width="6.42578125" style="10" customWidth="1"/>
+    <col min="4" max="4" width="35.7109375" style="10" customWidth="1"/>
     <col min="5" max="5" width="21" style="10" customWidth="1"/>
-    <col min="6" max="7" width="5.88671875" style="10" customWidth="1"/>
-    <col min="8" max="8" width="6.33203125" style="10" customWidth="1"/>
+    <col min="6" max="7" width="5.85546875" style="10" customWidth="1"/>
+    <col min="8" max="8" width="6.28515625" style="10" customWidth="1"/>
     <col min="9" max="9" width="6" style="10" customWidth="1"/>
-    <col min="10" max="10" width="6.44140625" style="10" customWidth="1"/>
-    <col min="11" max="18" width="5.44140625" style="10" customWidth="1"/>
-    <col min="19" max="19" width="4.33203125" style="10" customWidth="1"/>
+    <col min="10" max="10" width="6.42578125" style="10" customWidth="1"/>
+    <col min="11" max="18" width="5.42578125" style="10" customWidth="1"/>
+    <col min="19" max="19" width="4.28515625" style="10" customWidth="1"/>
     <col min="20" max="20" width="3" style="10" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="6.44140625" style="10" customWidth="1"/>
+    <col min="21" max="21" width="6.42578125" style="10" customWidth="1"/>
     <col min="22" max="22" width="11" style="10" customWidth="1"/>
-    <col min="23" max="24" width="29.33203125" style="10" customWidth="1"/>
-    <col min="25" max="16384" width="10.88671875" style="10"/>
+    <col min="23" max="24" width="29.28515625" style="10" customWidth="1"/>
+    <col min="25" max="16384" width="10.85546875" style="10"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:24" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="68" t="s">
+    <row r="2" spans="1:24" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="67" t="s">
         <v>32</v>
       </c>
-      <c r="B2" s="61" t="s">
+      <c r="B2" s="26" t="s">
         <v>54</v>
       </c>
-      <c r="C2" s="66" t="s">
+      <c r="C2" s="65" t="s">
         <v>53</v>
       </c>
-      <c r="D2" s="44" t="s">
+      <c r="D2" s="29" t="s">
         <v>50</v>
       </c>
-      <c r="E2" s="44" t="s">
+      <c r="E2" s="29" t="s">
         <v>48</v>
       </c>
-      <c r="F2" s="65" t="s">
+      <c r="F2" s="69" t="s">
         <v>55</v>
       </c>
-      <c r="G2" s="59"/>
-      <c r="H2" s="59"/>
-      <c r="I2" s="59"/>
-      <c r="J2" s="59"/>
-      <c r="K2" s="59"/>
-      <c r="L2" s="59"/>
-      <c r="M2" s="59"/>
-      <c r="N2" s="59"/>
-      <c r="O2" s="59"/>
-      <c r="P2" s="59"/>
-      <c r="Q2" s="59"/>
-      <c r="R2" s="59"/>
-      <c r="S2" s="59"/>
-      <c r="T2" s="59"/>
-      <c r="U2" s="60"/>
+      <c r="G2" s="45"/>
+      <c r="H2" s="45"/>
+      <c r="I2" s="45"/>
+      <c r="J2" s="45"/>
+      <c r="K2" s="45"/>
+      <c r="L2" s="45"/>
+      <c r="M2" s="45"/>
+      <c r="N2" s="45"/>
+      <c r="O2" s="45"/>
+      <c r="P2" s="45"/>
+      <c r="Q2" s="45"/>
+      <c r="R2" s="45"/>
+      <c r="S2" s="45"/>
+      <c r="T2" s="45"/>
+      <c r="U2" s="46"/>
       <c r="V2" s="16"/>
-      <c r="W2" s="44" t="s">
+      <c r="W2" s="29" t="s">
         <v>71</v>
       </c>
-      <c r="X2" s="44" t="s">
+      <c r="X2" s="29" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="3" spans="1:24" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="68"/>
-      <c r="B3" s="61"/>
-      <c r="C3" s="66"/>
-      <c r="D3" s="45"/>
-      <c r="E3" s="45"/>
-      <c r="F3" s="58" t="s">
+    <row r="3" spans="1:24" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="67"/>
+      <c r="B3" s="26"/>
+      <c r="C3" s="65"/>
+      <c r="D3" s="30"/>
+      <c r="E3" s="30"/>
+      <c r="F3" s="44" t="s">
         <v>49</v>
       </c>
-      <c r="G3" s="47"/>
-      <c r="H3" s="47"/>
-      <c r="I3" s="47"/>
-      <c r="J3" s="47"/>
-      <c r="K3" s="47"/>
-      <c r="L3" s="47"/>
-      <c r="M3" s="47"/>
-      <c r="N3" s="48"/>
-      <c r="O3" s="49" t="s">
+      <c r="G3" s="33"/>
+      <c r="H3" s="33"/>
+      <c r="I3" s="33"/>
+      <c r="J3" s="33"/>
+      <c r="K3" s="33"/>
+      <c r="L3" s="33"/>
+      <c r="M3" s="33"/>
+      <c r="N3" s="34"/>
+      <c r="O3" s="35" t="s">
         <v>44</v>
       </c>
-      <c r="P3" s="50"/>
-      <c r="Q3" s="50"/>
-      <c r="R3" s="50"/>
-      <c r="S3" s="50"/>
-      <c r="T3" s="50"/>
-      <c r="U3" s="51"/>
-      <c r="V3" s="55" t="s">
+      <c r="P3" s="36"/>
+      <c r="Q3" s="36"/>
+      <c r="R3" s="36"/>
+      <c r="S3" s="36"/>
+      <c r="T3" s="36"/>
+      <c r="U3" s="37"/>
+      <c r="V3" s="41" t="s">
         <v>67</v>
       </c>
-      <c r="W3" s="45"/>
-      <c r="X3" s="45"/>
-    </row>
-    <row r="4" spans="1:24" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="69"/>
-      <c r="B4" s="61"/>
-      <c r="C4" s="66"/>
-      <c r="D4" s="45"/>
-      <c r="E4" s="45"/>
-      <c r="F4" s="58" t="s">
+      <c r="W3" s="30"/>
+      <c r="X3" s="30"/>
+    </row>
+    <row r="4" spans="1:24" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="68"/>
+      <c r="B4" s="26"/>
+      <c r="C4" s="65"/>
+      <c r="D4" s="30"/>
+      <c r="E4" s="30"/>
+      <c r="F4" s="44" t="s">
         <v>45</v>
       </c>
-      <c r="G4" s="47"/>
-      <c r="H4" s="47"/>
-      <c r="I4" s="48"/>
-      <c r="J4" s="58" t="s">
+      <c r="G4" s="33"/>
+      <c r="H4" s="33"/>
+      <c r="I4" s="34"/>
+      <c r="J4" s="44" t="s">
         <v>47</v>
       </c>
-      <c r="K4" s="47"/>
-      <c r="L4" s="48"/>
-      <c r="M4" s="58" t="s">
+      <c r="K4" s="33"/>
+      <c r="L4" s="34"/>
+      <c r="M4" s="44" t="s">
         <v>46</v>
       </c>
-      <c r="N4" s="48"/>
-      <c r="O4" s="52"/>
-      <c r="P4" s="53"/>
-      <c r="Q4" s="53"/>
-      <c r="R4" s="53"/>
-      <c r="S4" s="53"/>
-      <c r="T4" s="53"/>
-      <c r="U4" s="54"/>
-      <c r="V4" s="56"/>
-      <c r="W4" s="45"/>
-      <c r="X4" s="45"/>
-    </row>
-    <row r="5" spans="1:24" ht="113.4" x14ac:dyDescent="0.25">
+      <c r="N4" s="34"/>
+      <c r="O4" s="38"/>
+      <c r="P4" s="39"/>
+      <c r="Q4" s="39"/>
+      <c r="R4" s="39"/>
+      <c r="S4" s="39"/>
+      <c r="T4" s="39"/>
+      <c r="U4" s="40"/>
+      <c r="V4" s="42"/>
+      <c r="W4" s="30"/>
+      <c r="X4" s="30"/>
+    </row>
+    <row r="5" spans="1:24" ht="114" x14ac:dyDescent="0.2">
       <c r="A5" s="15" t="s">
         <v>89</v>
       </c>
-      <c r="B5" s="61"/>
-      <c r="C5" s="67"/>
-      <c r="D5" s="46"/>
-      <c r="E5" s="46"/>
+      <c r="B5" s="26"/>
+      <c r="C5" s="66"/>
+      <c r="D5" s="31"/>
+      <c r="E5" s="31"/>
       <c r="F5" s="11" t="s">
         <v>56</v>
       </c>
@@ -5197,11 +5197,11 @@
       <c r="U5" s="11" t="s">
         <v>81</v>
       </c>
-      <c r="V5" s="57"/>
-      <c r="W5" s="46"/>
-      <c r="X5" s="46"/>
-    </row>
-    <row r="6" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="V5" s="43"/>
+      <c r="W5" s="31"/>
+      <c r="X5" s="31"/>
+    </row>
+    <row r="6" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A6" s="70"/>
       <c r="B6" s="9"/>
       <c r="C6" s="9"/>
@@ -5227,7 +5227,7 @@
       <c r="W6" s="9"/>
       <c r="X6" s="9"/>
     </row>
-    <row r="7" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A7" s="71"/>
       <c r="B7" s="9"/>
       <c r="C7" s="9"/>
@@ -5253,7 +5253,7 @@
       <c r="W7" s="9"/>
       <c r="X7" s="9"/>
     </row>
-    <row r="8" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A8" s="71"/>
       <c r="B8" s="9"/>
       <c r="C8" s="9"/>
@@ -5279,7 +5279,7 @@
       <c r="W8" s="9"/>
       <c r="X8" s="9"/>
     </row>
-    <row r="9" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A9" s="71"/>
       <c r="B9" s="9"/>
       <c r="C9" s="9"/>
@@ -5305,7 +5305,7 @@
       <c r="W9" s="9"/>
       <c r="X9" s="9"/>
     </row>
-    <row r="10" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A10" s="71"/>
       <c r="B10" s="9"/>
       <c r="C10" s="9"/>
@@ -5331,7 +5331,7 @@
       <c r="W10" s="9"/>
       <c r="X10" s="9"/>
     </row>
-    <row r="11" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A11" s="71"/>
       <c r="B11" s="9"/>
       <c r="C11" s="9"/>
@@ -5357,7 +5357,7 @@
       <c r="W11" s="9"/>
       <c r="X11" s="9"/>
     </row>
-    <row r="12" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A12" s="71"/>
       <c r="B12" s="9"/>
       <c r="C12" s="9"/>
@@ -5383,7 +5383,7 @@
       <c r="W12" s="9"/>
       <c r="X12" s="9"/>
     </row>
-    <row r="13" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A13" s="71"/>
       <c r="B13" s="9"/>
       <c r="C13" s="9"/>
@@ -5409,7 +5409,7 @@
       <c r="W13" s="9"/>
       <c r="X13" s="9"/>
     </row>
-    <row r="14" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A14" s="71"/>
       <c r="B14" s="9"/>
       <c r="C14" s="9"/>
@@ -5435,7 +5435,7 @@
       <c r="W14" s="9"/>
       <c r="X14" s="9"/>
     </row>
-    <row r="15" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A15" s="71"/>
       <c r="B15" s="9"/>
       <c r="C15" s="9"/>
@@ -5461,7 +5461,7 @@
       <c r="W15" s="9"/>
       <c r="X15" s="9"/>
     </row>
-    <row r="16" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A16" s="71"/>
       <c r="B16" s="9"/>
       <c r="C16" s="9"/>
@@ -5487,7 +5487,7 @@
       <c r="W16" s="12"/>
       <c r="X16" s="12"/>
     </row>
-    <row r="17" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A17" s="71"/>
       <c r="B17" s="9"/>
       <c r="C17" s="9"/>
@@ -5513,7 +5513,7 @@
       <c r="W17" s="12"/>
       <c r="X17" s="12"/>
     </row>
-    <row r="18" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A18" s="72"/>
       <c r="B18" s="9"/>
       <c r="C18" s="9"/>
@@ -5539,41 +5539,50 @@
       <c r="W18" s="12"/>
       <c r="X18" s="12"/>
     </row>
-    <row r="29" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A29" s="62" t="s">
+    <row r="29" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A29" s="27" t="s">
         <v>92</v>
       </c>
-      <c r="B29" s="62"/>
-      <c r="C29" s="62"/>
-      <c r="D29" s="62"/>
-      <c r="E29" s="63"/>
-    </row>
-    <row r="30" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A30" s="62"/>
-      <c r="B30" s="62"/>
-      <c r="C30" s="62"/>
-      <c r="D30" s="62"/>
-      <c r="E30" s="63"/>
-    </row>
-    <row r="31" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A31" s="62" t="s">
+      <c r="B29" s="27"/>
+      <c r="C29" s="27"/>
+      <c r="D29" s="27"/>
+      <c r="E29" s="28"/>
+    </row>
+    <row r="30" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A30" s="27"/>
+      <c r="B30" s="27"/>
+      <c r="C30" s="27"/>
+      <c r="D30" s="27"/>
+      <c r="E30" s="28"/>
+    </row>
+    <row r="31" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A31" s="27" t="s">
         <v>91</v>
       </c>
-      <c r="B31" s="62"/>
-      <c r="C31" s="62"/>
-      <c r="D31" s="62"/>
-      <c r="E31" s="63"/>
-    </row>
-    <row r="32" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A32" s="62"/>
-      <c r="B32" s="62"/>
-      <c r="C32" s="62"/>
-      <c r="D32" s="62"/>
-      <c r="E32" s="63"/>
+      <c r="B31" s="27"/>
+      <c r="C31" s="27"/>
+      <c r="D31" s="27"/>
+      <c r="E31" s="28"/>
+    </row>
+    <row r="32" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A32" s="27"/>
+      <c r="B32" s="27"/>
+      <c r="C32" s="27"/>
+      <c r="D32" s="27"/>
+      <c r="E32" s="28"/>
     </row>
   </sheetData>
   <dataConsolidate/>
   <mergeCells count="19">
+    <mergeCell ref="X2:X5"/>
+    <mergeCell ref="F3:N3"/>
+    <mergeCell ref="O3:U4"/>
+    <mergeCell ref="V3:V5"/>
+    <mergeCell ref="F4:I4"/>
+    <mergeCell ref="J4:L4"/>
+    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="W2:W5"/>
+    <mergeCell ref="F2:U2"/>
     <mergeCell ref="B2:B5"/>
     <mergeCell ref="A29:D30"/>
     <mergeCell ref="E29:E30"/>
@@ -5584,15 +5593,6 @@
     <mergeCell ref="E2:E5"/>
     <mergeCell ref="A6:A18"/>
     <mergeCell ref="A2:A4"/>
-    <mergeCell ref="X2:X5"/>
-    <mergeCell ref="F3:N3"/>
-    <mergeCell ref="O3:U4"/>
-    <mergeCell ref="V3:V5"/>
-    <mergeCell ref="F4:I4"/>
-    <mergeCell ref="J4:L4"/>
-    <mergeCell ref="M4:N4"/>
-    <mergeCell ref="W2:W5"/>
-    <mergeCell ref="F2:U2"/>
   </mergeCells>
   <conditionalFormatting sqref="U6:U18">
     <cfRule type="containsText" dxfId="0" priority="1" stopIfTrue="1" operator="containsText" text="SI">
@@ -5646,15 +5646,15 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A2:D18"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="36.5546875" customWidth="1"/>
-    <col min="2" max="2" width="20.6640625" customWidth="1"/>
-    <col min="3" max="3" width="7.33203125" customWidth="1"/>
-    <col min="4" max="4" width="38.6640625" customWidth="1"/>
+    <col min="1" max="1" width="36.5703125" customWidth="1"/>
+    <col min="2" max="2" width="20.7109375" customWidth="1"/>
+    <col min="3" max="3" width="7.28515625" customWidth="1"/>
+    <col min="4" max="4" width="38.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B2" s="21" t="s">
         <v>83</v>
       </c>
@@ -5662,7 +5662,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="22">
         <v>1</v>
       </c>
@@ -5676,7 +5676,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="22">
         <v>2</v>
       </c>
@@ -5690,7 +5690,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="22">
         <v>3</v>
       </c>
@@ -5704,7 +5704,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="22">
         <v>4</v>
       </c>
@@ -5718,7 +5718,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="22">
         <v>5</v>
       </c>
@@ -5732,7 +5732,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="22">
         <v>6</v>
       </c>
@@ -5746,7 +5746,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C9" s="17">
         <v>7</v>
       </c>
@@ -5754,7 +5754,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C10" s="17">
         <v>8</v>
       </c>
@@ -5762,7 +5762,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C11" s="17">
         <v>9</v>
       </c>
@@ -5770,7 +5770,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C12" s="17">
         <v>10</v>
       </c>
@@ -5778,7 +5778,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C13" s="17">
         <v>11</v>
       </c>
@@ -5786,7 +5786,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C14" s="17">
         <v>12</v>
       </c>
@@ -5794,7 +5794,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C15" s="17">
         <v>13</v>
       </c>
@@ -5802,7 +5802,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C16" s="17">
         <v>14</v>
       </c>
@@ -5810,7 +5810,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="17" spans="3:4" x14ac:dyDescent="0.3">
+    <row r="17" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C17" s="17">
         <v>15</v>
       </c>
@@ -5818,7 +5818,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="18" spans="3:4" x14ac:dyDescent="0.3">
+    <row r="18" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C18" s="17">
         <v>16</v>
       </c>

</xml_diff>

<commit_message>
Terminacion de documentos SASISOPA
</commit_message>
<xml_diff>
--- a/sasisopa-machotes/sasisopa-machotes/F-02-02_Matriz_de_Identificación_de_Aspectos_e_Impactos_Ambientales.xlsx
+++ b/sasisopa-machotes/sasisopa-machotes/F-02-02_Matriz_de_Identificación_de_Aspectos_e_Impactos_Ambientales.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/01dae4c2401b18f1/Escritorio/portal-tecnocontrol-main GIt/portal-tecnocontrol/sasisopa-machotes/sasisopa-machotes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{511E3075-E7BB-4278-9A7A-1E44DF908B4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{31C79D52-B758-4EB3-935E-C3DEF4D84079}"/>
+  <xr:revisionPtr revIDLastSave="61" documentId="13_ncr:1_{511E3075-E7BB-4278-9A7A-1E44DF908B4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2FFD8456-59CF-482D-B891-002E85419BD6}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ANEXO 1" sheetId="2" r:id="rId1"/>
@@ -275,7 +275,7 @@
     <author>SUMMX</author>
   </authors>
   <commentList>
-    <comment ref="X2" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0300-000001000000}">
+    <comment ref="X6" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0300-000001000000}">
       <text>
         <r>
           <rPr>
@@ -300,7 +300,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="O5" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0300-000002000000}">
+    <comment ref="O9" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0300-000002000000}">
       <text>
         <r>
           <rPr>
@@ -316,7 +316,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="P5" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0300-000003000000}">
+    <comment ref="P9" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0300-000003000000}">
       <text>
         <r>
           <rPr>
@@ -332,7 +332,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Q5" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0300-000004000000}">
+    <comment ref="Q9" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0300-000004000000}">
       <text>
         <r>
           <rPr>
@@ -348,7 +348,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="R5" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0300-000005000000}">
+    <comment ref="R9" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0300-000005000000}">
       <text>
         <r>
           <rPr>
@@ -363,7 +363,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="S5" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0300-000006000000}">
+    <comment ref="S9" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0300-000006000000}">
       <text>
         <r>
           <rPr>
@@ -388,7 +388,7 @@
     <author>SUMMX</author>
   </authors>
   <commentList>
-    <comment ref="X2" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0400-000001000000}">
+    <comment ref="X6" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0400-000001000000}">
       <text>
         <r>
           <rPr>
@@ -413,7 +413,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="O5" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0400-000002000000}">
+    <comment ref="O9" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0400-000002000000}">
       <text>
         <r>
           <rPr>
@@ -429,7 +429,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="P5" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0400-000003000000}">
+    <comment ref="P9" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0400-000003000000}">
       <text>
         <r>
           <rPr>
@@ -445,7 +445,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Q5" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0400-000004000000}">
+    <comment ref="Q9" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0400-000004000000}">
       <text>
         <r>
           <rPr>
@@ -461,7 +461,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="R5" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0400-000005000000}">
+    <comment ref="R9" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0400-000005000000}">
       <text>
         <r>
           <rPr>
@@ -476,7 +476,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="S5" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0400-000006000000}">
+    <comment ref="S9" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0400-000006000000}">
       <text>
         <r>
           <rPr>
@@ -496,7 +496,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="203" uniqueCount="100">
   <si>
     <t>Con relación a la magnitud del impacto</t>
   </si>
@@ -784,6 +784,70 @@
   </si>
   <si>
     <t>COMPONENTES</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>SUPERSERVICIO CUATRO CAMINOS S.A DE C.V</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+TÍTULO
+MATRIZ DE ASPECTOS E IMPACTOS AMBIENTALES
+Revisión Número: 0</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>CLAVE: F-02-02           
+       FECHA DE EMISIÓN:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>01/03/2019</t>
+    </r>
+  </si>
+  <si>
+    <t>LOGO</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>SUPERSERVICIO CUATRO CAMINOS S.A DE C.V</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+TÍTULO
+Matriz de Identificación de Aspectos Ambientales 
+Revisión Número: 0</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -794,7 +858,7 @@
     <numFmt numFmtId="164" formatCode="_ [$€-2]\ * #,##0.00_ ;_ [$€-2]\ * \-#,##0.00_ ;_ [$€-2]\ * &quot;-&quot;??_ "/>
     <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd;@"/>
   </numFmts>
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -909,8 +973,14 @@
       <name val="Arial Narrow"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -945,6 +1015,12 @@
       <patternFill patternType="lightGray">
         <fgColor theme="3" tint="0.39994506668294322"/>
         <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -1255,7 +1331,7 @@
       <alignment horizontal="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="73">
+  <cellXfs count="82">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1328,145 +1404,172 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="13" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="13" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2200,7 +2303,7 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>190501</xdr:colOff>
-      <xdr:row>21</xdr:row>
+      <xdr:row>25</xdr:row>
       <xdr:rowOff>68036</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="3837214" cy="1346516"/>
@@ -2307,7 +2410,7 @@
     <xdr:from>
       <xdr:col>16</xdr:col>
       <xdr:colOff>108857</xdr:colOff>
-      <xdr:row>20</xdr:row>
+      <xdr:row>24</xdr:row>
       <xdr:rowOff>23813</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="3837214" cy="1346516"/>
@@ -2430,7 +2533,7 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>285751</xdr:colOff>
-      <xdr:row>20</xdr:row>
+      <xdr:row>24</xdr:row>
       <xdr:rowOff>44224</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="3837214" cy="1346516"/>
@@ -2537,7 +2640,7 @@
     <xdr:from>
       <xdr:col>3</xdr:col>
       <xdr:colOff>2287701</xdr:colOff>
-      <xdr:row>20</xdr:row>
+      <xdr:row>24</xdr:row>
       <xdr:rowOff>35719</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="3837214" cy="1346516"/>
@@ -2652,6 +2755,10 @@
     <xdr:clientData/>
   </xdr:oneCellAnchor>
 </xdr:wsDr>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2988,27 +3095,27 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="49" t="s">
+      <c r="A1" s="61" t="s">
         <v>93</v>
       </c>
-      <c r="B1" s="49"/>
-      <c r="C1" s="49"/>
-      <c r="D1" s="49"/>
+      <c r="B1" s="61"/>
+      <c r="C1" s="61"/>
+      <c r="D1" s="61"/>
     </row>
     <row r="2" spans="1:4" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="58" t="s">
+      <c r="A2" s="72" t="s">
         <v>27</v>
       </c>
       <c r="B2" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="C2" s="52" t="s">
+      <c r="C2" s="64" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="52"/>
+      <c r="D2" s="64"/>
     </row>
     <row r="3" spans="1:4" ht="41.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="58"/>
+      <c r="A3" s="72"/>
       <c r="B3" s="1">
         <v>1</v>
       </c>
@@ -3020,7 +3127,7 @@
       </c>
     </row>
     <row r="4" spans="1:4" ht="42.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="58"/>
+      <c r="A4" s="72"/>
       <c r="B4" s="1">
         <v>2</v>
       </c>
@@ -3032,7 +3139,7 @@
       </c>
     </row>
     <row r="5" spans="1:4" ht="41.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="58"/>
+      <c r="A5" s="72"/>
       <c r="B5" s="1">
         <v>3</v>
       </c>
@@ -3044,17 +3151,17 @@
       </c>
     </row>
     <row r="6" spans="1:4" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="58"/>
+      <c r="A6" s="72"/>
       <c r="B6" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="C6" s="52" t="s">
+      <c r="C6" s="64" t="s">
         <v>7</v>
       </c>
-      <c r="D6" s="52"/>
+      <c r="D6" s="64"/>
     </row>
     <row r="7" spans="1:4" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="58"/>
+      <c r="A7" s="72"/>
       <c r="B7" s="1">
         <v>1</v>
       </c>
@@ -3066,7 +3173,7 @@
       </c>
     </row>
     <row r="8" spans="1:4" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="58"/>
+      <c r="A8" s="72"/>
       <c r="B8" s="1">
         <v>2</v>
       </c>
@@ -3078,7 +3185,7 @@
       </c>
     </row>
     <row r="9" spans="1:4" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="58"/>
+      <c r="A9" s="72"/>
       <c r="B9" s="1">
         <v>3</v>
       </c>
@@ -3090,17 +3197,17 @@
       </c>
     </row>
     <row r="10" spans="1:4" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="58"/>
+      <c r="A10" s="72"/>
       <c r="B10" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="C10" s="50" t="s">
+      <c r="C10" s="62" t="s">
         <v>14</v>
       </c>
-      <c r="D10" s="51"/>
+      <c r="D10" s="63"/>
     </row>
     <row r="11" spans="1:4" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="58"/>
+      <c r="A11" s="72"/>
       <c r="B11" s="1">
         <v>1</v>
       </c>
@@ -3112,7 +3219,7 @@
       </c>
     </row>
     <row r="12" spans="1:4" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="58"/>
+      <c r="A12" s="72"/>
       <c r="B12" s="1">
         <v>2</v>
       </c>
@@ -3124,7 +3231,7 @@
       </c>
     </row>
     <row r="13" spans="1:4" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="58"/>
+      <c r="A13" s="72"/>
       <c r="B13" s="1">
         <v>3</v>
       </c>
@@ -3136,114 +3243,113 @@
       </c>
     </row>
     <row r="14" spans="1:4" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="57"/>
-      <c r="C14" s="57"/>
-      <c r="D14" s="57"/>
+      <c r="B14" s="71"/>
+      <c r="C14" s="71"/>
+      <c r="D14" s="71"/>
     </row>
     <row r="15" spans="1:4" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="53" t="s">
+      <c r="A15" s="67" t="s">
         <v>28</v>
       </c>
       <c r="B15" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="C15" s="52" t="s">
+      <c r="C15" s="64" t="s">
         <v>68</v>
       </c>
-      <c r="D15" s="52"/>
+      <c r="D15" s="64"/>
     </row>
     <row r="16" spans="1:4" ht="19.899999999999999" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="54"/>
+      <c r="A16" s="68"/>
       <c r="B16" s="7">
         <v>0</v>
       </c>
-      <c r="C16" s="62" t="s">
+      <c r="C16" s="76" t="s">
         <v>22</v>
       </c>
-      <c r="D16" s="62"/>
+      <c r="D16" s="76"/>
     </row>
     <row r="17" spans="1:4" ht="19.899999999999999" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="54"/>
+      <c r="A17" s="68"/>
       <c r="B17" s="7">
         <v>10</v>
       </c>
-      <c r="C17" s="63" t="s">
+      <c r="C17" s="77" t="s">
         <v>23</v>
       </c>
-      <c r="D17" s="64"/>
+      <c r="D17" s="78"/>
     </row>
     <row r="18" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="54"/>
+      <c r="A18" s="68"/>
       <c r="B18" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="C18" s="50" t="s">
+      <c r="C18" s="62" t="s">
         <v>52</v>
       </c>
-      <c r="D18" s="51"/>
+      <c r="D18" s="63"/>
     </row>
     <row r="19" spans="1:4" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="54"/>
+      <c r="A19" s="68"/>
       <c r="B19" s="7">
         <v>0</v>
       </c>
-      <c r="C19" s="56" t="s">
+      <c r="C19" s="70" t="s">
         <v>21</v>
       </c>
-      <c r="D19" s="56"/>
+      <c r="D19" s="70"/>
     </row>
     <row r="20" spans="1:4" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="55"/>
+      <c r="A20" s="69"/>
       <c r="B20" s="7">
         <v>10</v>
       </c>
-      <c r="C20" s="56" t="s">
+      <c r="C20" s="70" t="s">
         <v>30</v>
       </c>
-      <c r="D20" s="56"/>
+      <c r="D20" s="70"/>
     </row>
     <row r="22" spans="1:4" ht="13.5" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="23" spans="1:4" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="50" t="s">
+      <c r="A23" s="62" t="s">
         <v>77</v>
       </c>
-      <c r="B23" s="61"/>
-      <c r="C23" s="61"/>
-      <c r="D23" s="51"/>
+      <c r="B23" s="75"/>
+      <c r="C23" s="75"/>
+      <c r="D23" s="63"/>
     </row>
     <row r="24" spans="1:4" ht="73.900000000000006" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="50" t="s">
+      <c r="A24" s="62" t="s">
         <v>25</v>
       </c>
-      <c r="B24" s="51"/>
-      <c r="C24" s="59" t="s">
+      <c r="B24" s="63"/>
+      <c r="C24" s="73" t="s">
         <v>73</v>
       </c>
-      <c r="D24" s="60"/>
+      <c r="D24" s="74"/>
     </row>
     <row r="25" spans="1:4" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="50" t="s">
+      <c r="A25" s="62" t="s">
         <v>26</v>
       </c>
-      <c r="B25" s="51"/>
-      <c r="C25" s="47" t="s">
+      <c r="B25" s="63"/>
+      <c r="C25" s="65" t="s">
         <v>74</v>
       </c>
-      <c r="D25" s="48"/>
+      <c r="D25" s="66"/>
     </row>
     <row r="26" spans="1:4" ht="44.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="50" t="s">
+      <c r="A26" s="62" t="s">
         <v>24</v>
       </c>
-      <c r="B26" s="51"/>
-      <c r="C26" s="47" t="s">
+      <c r="B26" s="63"/>
+      <c r="C26" s="65" t="s">
         <v>72</v>
       </c>
-      <c r="D26" s="48"/>
+      <c r="D26" s="66"/>
     </row>
   </sheetData>
   <mergeCells count="20">
-    <mergeCell ref="C16:D16"/>
     <mergeCell ref="C17:D17"/>
     <mergeCell ref="C18:D18"/>
     <mergeCell ref="C19:D19"/>
@@ -3263,6 +3369,7 @@
     <mergeCell ref="A25:B25"/>
     <mergeCell ref="C24:D24"/>
     <mergeCell ref="A23:D23"/>
+    <mergeCell ref="C16:D16"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1.0119047619047619" bottom="1" header="0.3" footer="0.3"/>
@@ -3306,116 +3413,116 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:23" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="81" t="s">
         <v>32</v>
       </c>
-      <c r="B1" s="26" t="s">
+      <c r="B1" s="38" t="s">
         <v>54</v>
       </c>
-      <c r="C1" s="26" t="s">
+      <c r="C1" s="38" t="s">
         <v>53</v>
       </c>
-      <c r="D1" s="29" t="s">
+      <c r="D1" s="41" t="s">
         <v>50</v>
       </c>
-      <c r="E1" s="29" t="s">
+      <c r="E1" s="41" t="s">
         <v>48</v>
       </c>
-      <c r="F1" s="45" t="s">
+      <c r="F1" s="59" t="s">
         <v>55</v>
       </c>
-      <c r="G1" s="45"/>
-      <c r="H1" s="45"/>
-      <c r="I1" s="45"/>
-      <c r="J1" s="45"/>
-      <c r="K1" s="45"/>
-      <c r="L1" s="45"/>
-      <c r="M1" s="45"/>
-      <c r="N1" s="45"/>
-      <c r="O1" s="45"/>
-      <c r="P1" s="45"/>
-      <c r="Q1" s="45"/>
-      <c r="R1" s="45"/>
-      <c r="S1" s="45"/>
-      <c r="T1" s="46"/>
+      <c r="G1" s="59"/>
+      <c r="H1" s="59"/>
+      <c r="I1" s="59"/>
+      <c r="J1" s="59"/>
+      <c r="K1" s="59"/>
+      <c r="L1" s="59"/>
+      <c r="M1" s="59"/>
+      <c r="N1" s="59"/>
+      <c r="O1" s="59"/>
+      <c r="P1" s="59"/>
+      <c r="Q1" s="59"/>
+      <c r="R1" s="59"/>
+      <c r="S1" s="59"/>
+      <c r="T1" s="60"/>
       <c r="U1" s="16"/>
-      <c r="V1" s="29" t="s">
+      <c r="V1" s="41" t="s">
         <v>71</v>
       </c>
-      <c r="W1" s="29" t="s">
+      <c r="W1" s="41" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="2" spans="1:23" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="32"/>
-      <c r="B2" s="26"/>
-      <c r="C2" s="26"/>
-      <c r="D2" s="30"/>
-      <c r="E2" s="30"/>
-      <c r="F2" s="33" t="s">
+      <c r="A2" s="81"/>
+      <c r="B2" s="38"/>
+      <c r="C2" s="38"/>
+      <c r="D2" s="42"/>
+      <c r="E2" s="42"/>
+      <c r="F2" s="47" t="s">
         <v>95</v>
       </c>
-      <c r="G2" s="33"/>
-      <c r="H2" s="33"/>
-      <c r="I2" s="33"/>
-      <c r="J2" s="33"/>
-      <c r="K2" s="33"/>
-      <c r="L2" s="33"/>
-      <c r="M2" s="34"/>
-      <c r="N2" s="35" t="s">
+      <c r="G2" s="47"/>
+      <c r="H2" s="47"/>
+      <c r="I2" s="47"/>
+      <c r="J2" s="47"/>
+      <c r="K2" s="47"/>
+      <c r="L2" s="47"/>
+      <c r="M2" s="48"/>
+      <c r="N2" s="49" t="s">
         <v>44</v>
       </c>
-      <c r="O2" s="36"/>
-      <c r="P2" s="36"/>
-      <c r="Q2" s="36"/>
-      <c r="R2" s="36"/>
-      <c r="S2" s="36"/>
-      <c r="T2" s="37"/>
-      <c r="U2" s="41" t="s">
+      <c r="O2" s="50"/>
+      <c r="P2" s="50"/>
+      <c r="Q2" s="50"/>
+      <c r="R2" s="50"/>
+      <c r="S2" s="50"/>
+      <c r="T2" s="51"/>
+      <c r="U2" s="55" t="s">
         <v>67</v>
       </c>
-      <c r="V2" s="30"/>
-      <c r="W2" s="30"/>
+      <c r="V2" s="42"/>
+      <c r="W2" s="42"/>
     </row>
     <row r="3" spans="1:23" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="32"/>
-      <c r="B3" s="26"/>
-      <c r="C3" s="26"/>
-      <c r="D3" s="30"/>
-      <c r="E3" s="30"/>
-      <c r="F3" s="33" t="s">
+      <c r="A3" s="81"/>
+      <c r="B3" s="38"/>
+      <c r="C3" s="38"/>
+      <c r="D3" s="42"/>
+      <c r="E3" s="42"/>
+      <c r="F3" s="47" t="s">
         <v>45</v>
       </c>
-      <c r="G3" s="33"/>
-      <c r="H3" s="34"/>
-      <c r="I3" s="44" t="s">
+      <c r="G3" s="47"/>
+      <c r="H3" s="48"/>
+      <c r="I3" s="46" t="s">
         <v>47</v>
       </c>
-      <c r="J3" s="33"/>
-      <c r="K3" s="34"/>
-      <c r="L3" s="44" t="s">
+      <c r="J3" s="47"/>
+      <c r="K3" s="48"/>
+      <c r="L3" s="46" t="s">
         <v>46</v>
       </c>
-      <c r="M3" s="34"/>
-      <c r="N3" s="38"/>
-      <c r="O3" s="39"/>
-      <c r="P3" s="39"/>
-      <c r="Q3" s="39"/>
-      <c r="R3" s="39"/>
-      <c r="S3" s="39"/>
-      <c r="T3" s="40"/>
-      <c r="U3" s="42"/>
-      <c r="V3" s="30"/>
-      <c r="W3" s="30"/>
+      <c r="M3" s="48"/>
+      <c r="N3" s="52"/>
+      <c r="O3" s="53"/>
+      <c r="P3" s="53"/>
+      <c r="Q3" s="53"/>
+      <c r="R3" s="53"/>
+      <c r="S3" s="53"/>
+      <c r="T3" s="54"/>
+      <c r="U3" s="56"/>
+      <c r="V3" s="42"/>
+      <c r="W3" s="42"/>
     </row>
     <row r="4" spans="1:23" ht="114" x14ac:dyDescent="0.2">
       <c r="A4" s="15" t="s">
         <v>86</v>
       </c>
-      <c r="B4" s="26"/>
-      <c r="C4" s="26"/>
-      <c r="D4" s="31"/>
-      <c r="E4" s="31"/>
+      <c r="B4" s="38"/>
+      <c r="C4" s="38"/>
+      <c r="D4" s="43"/>
+      <c r="E4" s="43"/>
       <c r="F4" s="11" t="s">
         <v>57</v>
       </c>
@@ -3461,9 +3568,9 @@
       <c r="T4" s="11" t="s">
         <v>81</v>
       </c>
-      <c r="U4" s="43"/>
-      <c r="V4" s="31"/>
-      <c r="W4" s="31"/>
+      <c r="U4" s="57"/>
+      <c r="V4" s="43"/>
+      <c r="W4" s="43"/>
     </row>
     <row r="5" spans="1:23" ht="122.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="24"/>
@@ -3741,36 +3848,36 @@
       <c r="W15" s="12"/>
     </row>
     <row r="24" spans="1:5" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="27" t="s">
+      <c r="A24" s="79" t="s">
         <v>94</v>
       </c>
-      <c r="B24" s="27"/>
-      <c r="C24" s="27"/>
-      <c r="D24" s="27"/>
-      <c r="E24" s="28"/>
+      <c r="B24" s="79"/>
+      <c r="C24" s="79"/>
+      <c r="D24" s="79"/>
+      <c r="E24" s="80"/>
     </row>
     <row r="25" spans="1:5" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="27"/>
-      <c r="B25" s="27"/>
-      <c r="C25" s="27"/>
-      <c r="D25" s="27"/>
-      <c r="E25" s="28"/>
+      <c r="A25" s="79"/>
+      <c r="B25" s="79"/>
+      <c r="C25" s="79"/>
+      <c r="D25" s="79"/>
+      <c r="E25" s="80"/>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A26" s="27" t="s">
+      <c r="A26" s="79" t="s">
         <v>91</v>
       </c>
-      <c r="B26" s="27"/>
-      <c r="C26" s="27"/>
-      <c r="D26" s="27"/>
-      <c r="E26" s="28"/>
+      <c r="B26" s="79"/>
+      <c r="C26" s="79"/>
+      <c r="D26" s="79"/>
+      <c r="E26" s="80"/>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A27" s="27"/>
-      <c r="B27" s="27"/>
-      <c r="C27" s="27"/>
-      <c r="D27" s="27"/>
-      <c r="E27" s="28"/>
+      <c r="A27" s="79"/>
+      <c r="B27" s="79"/>
+      <c r="C27" s="79"/>
+      <c r="D27" s="79"/>
+      <c r="E27" s="80"/>
     </row>
   </sheetData>
   <dataConsolidate/>
@@ -3872,119 +3979,119 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:24" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="67" t="s">
+      <c r="A2" s="44" t="s">
         <v>32</v>
       </c>
-      <c r="B2" s="26" t="s">
+      <c r="B2" s="38" t="s">
         <v>54</v>
       </c>
-      <c r="C2" s="65" t="s">
+      <c r="C2" s="39" t="s">
         <v>53</v>
       </c>
-      <c r="D2" s="29" t="s">
+      <c r="D2" s="41" t="s">
         <v>50</v>
       </c>
-      <c r="E2" s="29" t="s">
+      <c r="E2" s="41" t="s">
         <v>48</v>
       </c>
-      <c r="F2" s="69" t="s">
+      <c r="F2" s="58" t="s">
         <v>55</v>
       </c>
-      <c r="G2" s="45"/>
-      <c r="H2" s="45"/>
-      <c r="I2" s="45"/>
-      <c r="J2" s="45"/>
-      <c r="K2" s="45"/>
-      <c r="L2" s="45"/>
-      <c r="M2" s="45"/>
-      <c r="N2" s="45"/>
-      <c r="O2" s="45"/>
-      <c r="P2" s="45"/>
-      <c r="Q2" s="45"/>
-      <c r="R2" s="45"/>
-      <c r="S2" s="45"/>
-      <c r="T2" s="45"/>
-      <c r="U2" s="46"/>
+      <c r="G2" s="59"/>
+      <c r="H2" s="59"/>
+      <c r="I2" s="59"/>
+      <c r="J2" s="59"/>
+      <c r="K2" s="59"/>
+      <c r="L2" s="59"/>
+      <c r="M2" s="59"/>
+      <c r="N2" s="59"/>
+      <c r="O2" s="59"/>
+      <c r="P2" s="59"/>
+      <c r="Q2" s="59"/>
+      <c r="R2" s="59"/>
+      <c r="S2" s="59"/>
+      <c r="T2" s="59"/>
+      <c r="U2" s="60"/>
       <c r="V2" s="16"/>
-      <c r="W2" s="29" t="s">
+      <c r="W2" s="41" t="s">
         <v>71</v>
       </c>
-      <c r="X2" s="29" t="s">
+      <c r="X2" s="41" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="3" spans="1:24" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="67"/>
-      <c r="B3" s="26"/>
-      <c r="C3" s="65"/>
-      <c r="D3" s="30"/>
-      <c r="E3" s="30"/>
-      <c r="F3" s="44" t="s">
+      <c r="A3" s="44"/>
+      <c r="B3" s="38"/>
+      <c r="C3" s="39"/>
+      <c r="D3" s="42"/>
+      <c r="E3" s="42"/>
+      <c r="F3" s="46" t="s">
         <v>49</v>
       </c>
-      <c r="G3" s="33"/>
-      <c r="H3" s="33"/>
-      <c r="I3" s="33"/>
-      <c r="J3" s="33"/>
-      <c r="K3" s="33"/>
-      <c r="L3" s="33"/>
-      <c r="M3" s="33"/>
-      <c r="N3" s="34"/>
-      <c r="O3" s="35" t="s">
+      <c r="G3" s="47"/>
+      <c r="H3" s="47"/>
+      <c r="I3" s="47"/>
+      <c r="J3" s="47"/>
+      <c r="K3" s="47"/>
+      <c r="L3" s="47"/>
+      <c r="M3" s="47"/>
+      <c r="N3" s="48"/>
+      <c r="O3" s="49" t="s">
         <v>44</v>
       </c>
-      <c r="P3" s="36"/>
-      <c r="Q3" s="36"/>
-      <c r="R3" s="36"/>
-      <c r="S3" s="36"/>
-      <c r="T3" s="36"/>
-      <c r="U3" s="37"/>
-      <c r="V3" s="41" t="s">
+      <c r="P3" s="50"/>
+      <c r="Q3" s="50"/>
+      <c r="R3" s="50"/>
+      <c r="S3" s="50"/>
+      <c r="T3" s="50"/>
+      <c r="U3" s="51"/>
+      <c r="V3" s="55" t="s">
         <v>67</v>
       </c>
-      <c r="W3" s="30"/>
-      <c r="X3" s="30"/>
+      <c r="W3" s="42"/>
+      <c r="X3" s="42"/>
     </row>
     <row r="4" spans="1:24" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="68"/>
-      <c r="B4" s="26"/>
-      <c r="C4" s="65"/>
-      <c r="D4" s="30"/>
-      <c r="E4" s="30"/>
-      <c r="F4" s="44" t="s">
+      <c r="A4" s="45"/>
+      <c r="B4" s="38"/>
+      <c r="C4" s="39"/>
+      <c r="D4" s="42"/>
+      <c r="E4" s="42"/>
+      <c r="F4" s="46" t="s">
         <v>45</v>
       </c>
-      <c r="G4" s="33"/>
-      <c r="H4" s="33"/>
-      <c r="I4" s="34"/>
-      <c r="J4" s="44" t="s">
+      <c r="G4" s="47"/>
+      <c r="H4" s="47"/>
+      <c r="I4" s="48"/>
+      <c r="J4" s="46" t="s">
         <v>47</v>
       </c>
-      <c r="K4" s="33"/>
-      <c r="L4" s="34"/>
-      <c r="M4" s="44" t="s">
+      <c r="K4" s="47"/>
+      <c r="L4" s="48"/>
+      <c r="M4" s="46" t="s">
         <v>46</v>
       </c>
-      <c r="N4" s="34"/>
-      <c r="O4" s="38"/>
-      <c r="P4" s="39"/>
-      <c r="Q4" s="39"/>
-      <c r="R4" s="39"/>
-      <c r="S4" s="39"/>
-      <c r="T4" s="39"/>
-      <c r="U4" s="40"/>
-      <c r="V4" s="42"/>
-      <c r="W4" s="30"/>
-      <c r="X4" s="30"/>
+      <c r="N4" s="48"/>
+      <c r="O4" s="52"/>
+      <c r="P4" s="53"/>
+      <c r="Q4" s="53"/>
+      <c r="R4" s="53"/>
+      <c r="S4" s="53"/>
+      <c r="T4" s="53"/>
+      <c r="U4" s="54"/>
+      <c r="V4" s="56"/>
+      <c r="W4" s="42"/>
+      <c r="X4" s="42"/>
     </row>
     <row r="5" spans="1:24" ht="114" x14ac:dyDescent="0.2">
       <c r="A5" s="15" t="s">
         <v>87</v>
       </c>
-      <c r="B5" s="26"/>
-      <c r="C5" s="66"/>
-      <c r="D5" s="31"/>
-      <c r="E5" s="31"/>
+      <c r="B5" s="38"/>
+      <c r="C5" s="40"/>
+      <c r="D5" s="43"/>
+      <c r="E5" s="43"/>
       <c r="F5" s="11" t="s">
         <v>56</v>
       </c>
@@ -4033,9 +4140,9 @@
       <c r="U5" s="11" t="s">
         <v>81</v>
       </c>
-      <c r="V5" s="43"/>
-      <c r="W5" s="31"/>
-      <c r="X5" s="31"/>
+      <c r="V5" s="57"/>
+      <c r="W5" s="43"/>
+      <c r="X5" s="43"/>
     </row>
     <row r="6" spans="1:24" ht="87.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="24"/>
@@ -4272,36 +4379,36 @@
       <c r="X14" s="12"/>
     </row>
     <row r="26" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="27" t="s">
+      <c r="A26" s="79" t="s">
         <v>92</v>
       </c>
-      <c r="B26" s="27"/>
-      <c r="C26" s="27"/>
-      <c r="D26" s="27"/>
-      <c r="E26" s="28"/>
+      <c r="B26" s="79"/>
+      <c r="C26" s="79"/>
+      <c r="D26" s="79"/>
+      <c r="E26" s="80"/>
     </row>
     <row r="27" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="27"/>
-      <c r="B27" s="27"/>
-      <c r="C27" s="27"/>
-      <c r="D27" s="27"/>
-      <c r="E27" s="28"/>
+      <c r="A27" s="79"/>
+      <c r="B27" s="79"/>
+      <c r="C27" s="79"/>
+      <c r="D27" s="79"/>
+      <c r="E27" s="80"/>
     </row>
     <row r="28" spans="1:5" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="27" t="s">
+      <c r="A28" s="79" t="s">
         <v>91</v>
       </c>
-      <c r="B28" s="27"/>
-      <c r="C28" s="27"/>
-      <c r="D28" s="27"/>
-      <c r="E28" s="28"/>
+      <c r="B28" s="79"/>
+      <c r="C28" s="79"/>
+      <c r="D28" s="79"/>
+      <c r="E28" s="80"/>
     </row>
     <row r="29" spans="1:5" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="27"/>
-      <c r="B29" s="27"/>
-      <c r="C29" s="27"/>
-      <c r="D29" s="27"/>
-      <c r="E29" s="28"/>
+      <c r="A29" s="79"/>
+      <c r="B29" s="79"/>
+      <c r="C29" s="79"/>
+      <c r="D29" s="79"/>
+      <c r="E29" s="80"/>
     </row>
   </sheetData>
   <dataConsolidate/>
@@ -4381,7 +4488,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:X32"/>
+  <dimension ref="A1:X36"/>
   <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="31.85546875" style="10" customWidth="1"/>
@@ -4402,278 +4509,310 @@
     <col min="25" max="16384" width="10.85546875" style="10"/>
   </cols>
   <sheetData>
+    <row r="1" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A1" s="35" t="s">
+        <v>98</v>
+      </c>
+      <c r="B1" s="35"/>
+      <c r="C1" s="35"/>
+      <c r="D1" s="35"/>
+      <c r="E1" s="36" t="s">
+        <v>96</v>
+      </c>
+      <c r="F1" s="35"/>
+      <c r="G1" s="35"/>
+      <c r="H1" s="35"/>
+      <c r="I1" s="35"/>
+      <c r="J1" s="35"/>
+      <c r="K1" s="35"/>
+      <c r="L1" s="35"/>
+      <c r="M1" s="35"/>
+      <c r="N1" s="35"/>
+      <c r="O1" s="35"/>
+      <c r="P1" s="35"/>
+      <c r="Q1" s="35"/>
+      <c r="R1" s="35"/>
+      <c r="S1" s="35"/>
+      <c r="T1" s="35"/>
+      <c r="U1" s="35"/>
+      <c r="V1" s="32" t="s">
+        <v>97</v>
+      </c>
+      <c r="W1" s="33"/>
+      <c r="X1" s="33"/>
+    </row>
     <row r="2" spans="1:24" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="67" t="s">
+      <c r="A2" s="35"/>
+      <c r="B2" s="35"/>
+      <c r="C2" s="35"/>
+      <c r="D2" s="35"/>
+      <c r="E2" s="35"/>
+      <c r="F2" s="35"/>
+      <c r="G2" s="35"/>
+      <c r="H2" s="35"/>
+      <c r="I2" s="35"/>
+      <c r="J2" s="35"/>
+      <c r="K2" s="35"/>
+      <c r="L2" s="35"/>
+      <c r="M2" s="35"/>
+      <c r="N2" s="35"/>
+      <c r="O2" s="35"/>
+      <c r="P2" s="35"/>
+      <c r="Q2" s="35"/>
+      <c r="R2" s="35"/>
+      <c r="S2" s="35"/>
+      <c r="T2" s="35"/>
+      <c r="U2" s="35"/>
+      <c r="V2" s="33"/>
+      <c r="W2" s="33"/>
+      <c r="X2" s="33"/>
+    </row>
+    <row r="3" spans="1:24" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="35"/>
+      <c r="B3" s="35"/>
+      <c r="C3" s="35"/>
+      <c r="D3" s="35"/>
+      <c r="E3" s="35"/>
+      <c r="F3" s="35"/>
+      <c r="G3" s="35"/>
+      <c r="H3" s="35"/>
+      <c r="I3" s="35"/>
+      <c r="J3" s="35"/>
+      <c r="K3" s="35"/>
+      <c r="L3" s="35"/>
+      <c r="M3" s="35"/>
+      <c r="N3" s="35"/>
+      <c r="O3" s="35"/>
+      <c r="P3" s="35"/>
+      <c r="Q3" s="35"/>
+      <c r="R3" s="35"/>
+      <c r="S3" s="35"/>
+      <c r="T3" s="35"/>
+      <c r="U3" s="35"/>
+      <c r="V3" s="33"/>
+      <c r="W3" s="33"/>
+      <c r="X3" s="33"/>
+    </row>
+    <row r="4" spans="1:24" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="35"/>
+      <c r="B4" s="35"/>
+      <c r="C4" s="35"/>
+      <c r="D4" s="35"/>
+      <c r="E4" s="35"/>
+      <c r="F4" s="35"/>
+      <c r="G4" s="35"/>
+      <c r="H4" s="35"/>
+      <c r="I4" s="35"/>
+      <c r="J4" s="35"/>
+      <c r="K4" s="35"/>
+      <c r="L4" s="35"/>
+      <c r="M4" s="35"/>
+      <c r="N4" s="35"/>
+      <c r="O4" s="35"/>
+      <c r="P4" s="35"/>
+      <c r="Q4" s="35"/>
+      <c r="R4" s="35"/>
+      <c r="S4" s="35"/>
+      <c r="T4" s="35"/>
+      <c r="U4" s="35"/>
+      <c r="V4" s="33"/>
+      <c r="W4" s="33"/>
+      <c r="X4" s="33"/>
+    </row>
+    <row r="5" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A5" s="35"/>
+      <c r="B5" s="35"/>
+      <c r="C5" s="35"/>
+      <c r="D5" s="35"/>
+      <c r="E5" s="37"/>
+      <c r="F5" s="37"/>
+      <c r="G5" s="37"/>
+      <c r="H5" s="37"/>
+      <c r="I5" s="37"/>
+      <c r="J5" s="37"/>
+      <c r="K5" s="37"/>
+      <c r="L5" s="37"/>
+      <c r="M5" s="37"/>
+      <c r="N5" s="37"/>
+      <c r="O5" s="37"/>
+      <c r="P5" s="37"/>
+      <c r="Q5" s="37"/>
+      <c r="R5" s="37"/>
+      <c r="S5" s="37"/>
+      <c r="T5" s="37"/>
+      <c r="U5" s="37"/>
+      <c r="V5" s="34"/>
+      <c r="W5" s="34"/>
+      <c r="X5" s="34"/>
+    </row>
+    <row r="6" spans="1:24" ht="15" x14ac:dyDescent="0.2">
+      <c r="A6" s="44" t="s">
         <v>32</v>
       </c>
-      <c r="B2" s="26" t="s">
+      <c r="B6" s="38" t="s">
         <v>54</v>
       </c>
-      <c r="C2" s="65" t="s">
+      <c r="C6" s="39" t="s">
         <v>53</v>
       </c>
-      <c r="D2" s="29" t="s">
+      <c r="D6" s="41" t="s">
         <v>50</v>
       </c>
-      <c r="E2" s="29" t="s">
+      <c r="E6" s="41" t="s">
         <v>48</v>
       </c>
-      <c r="F2" s="69" t="s">
+      <c r="F6" s="58" t="s">
         <v>55</v>
       </c>
-      <c r="G2" s="45"/>
-      <c r="H2" s="45"/>
-      <c r="I2" s="45"/>
-      <c r="J2" s="45"/>
-      <c r="K2" s="45"/>
-      <c r="L2" s="45"/>
-      <c r="M2" s="45"/>
-      <c r="N2" s="45"/>
-      <c r="O2" s="45"/>
-      <c r="P2" s="45"/>
-      <c r="Q2" s="45"/>
-      <c r="R2" s="45"/>
-      <c r="S2" s="45"/>
-      <c r="T2" s="45"/>
-      <c r="U2" s="46"/>
-      <c r="V2" s="16"/>
-      <c r="W2" s="29" t="s">
+      <c r="G6" s="59"/>
+      <c r="H6" s="59"/>
+      <c r="I6" s="59"/>
+      <c r="J6" s="59"/>
+      <c r="K6" s="59"/>
+      <c r="L6" s="59"/>
+      <c r="M6" s="59"/>
+      <c r="N6" s="59"/>
+      <c r="O6" s="59"/>
+      <c r="P6" s="59"/>
+      <c r="Q6" s="59"/>
+      <c r="R6" s="59"/>
+      <c r="S6" s="59"/>
+      <c r="T6" s="59"/>
+      <c r="U6" s="60"/>
+      <c r="V6" s="16"/>
+      <c r="W6" s="41" t="s">
         <v>71</v>
       </c>
-      <c r="X2" s="29" t="s">
+      <c r="X6" s="41" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="3" spans="1:24" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="67"/>
-      <c r="B3" s="26"/>
-      <c r="C3" s="65"/>
-      <c r="D3" s="30"/>
-      <c r="E3" s="30"/>
-      <c r="F3" s="44" t="s">
+    <row r="7" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A7" s="44"/>
+      <c r="B7" s="38"/>
+      <c r="C7" s="39"/>
+      <c r="D7" s="42"/>
+      <c r="E7" s="42"/>
+      <c r="F7" s="46" t="s">
         <v>49</v>
       </c>
-      <c r="G3" s="33"/>
-      <c r="H3" s="33"/>
-      <c r="I3" s="33"/>
-      <c r="J3" s="33"/>
-      <c r="K3" s="33"/>
-      <c r="L3" s="33"/>
-      <c r="M3" s="33"/>
-      <c r="N3" s="34"/>
-      <c r="O3" s="35" t="s">
+      <c r="G7" s="47"/>
+      <c r="H7" s="47"/>
+      <c r="I7" s="47"/>
+      <c r="J7" s="47"/>
+      <c r="K7" s="47"/>
+      <c r="L7" s="47"/>
+      <c r="M7" s="47"/>
+      <c r="N7" s="48"/>
+      <c r="O7" s="49" t="s">
         <v>44</v>
       </c>
-      <c r="P3" s="36"/>
-      <c r="Q3" s="36"/>
-      <c r="R3" s="36"/>
-      <c r="S3" s="36"/>
-      <c r="T3" s="36"/>
-      <c r="U3" s="37"/>
-      <c r="V3" s="41" t="s">
+      <c r="P7" s="50"/>
+      <c r="Q7" s="50"/>
+      <c r="R7" s="50"/>
+      <c r="S7" s="50"/>
+      <c r="T7" s="50"/>
+      <c r="U7" s="51"/>
+      <c r="V7" s="55" t="s">
         <v>67</v>
       </c>
-      <c r="W3" s="30"/>
-      <c r="X3" s="30"/>
-    </row>
-    <row r="4" spans="1:24" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="68"/>
-      <c r="B4" s="26"/>
-      <c r="C4" s="65"/>
-      <c r="D4" s="30"/>
-      <c r="E4" s="30"/>
-      <c r="F4" s="44" t="s">
+      <c r="W7" s="42"/>
+      <c r="X7" s="42"/>
+    </row>
+    <row r="8" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A8" s="45"/>
+      <c r="B8" s="38"/>
+      <c r="C8" s="39"/>
+      <c r="D8" s="42"/>
+      <c r="E8" s="42"/>
+      <c r="F8" s="46" t="s">
         <v>45</v>
       </c>
-      <c r="G4" s="33"/>
-      <c r="H4" s="33"/>
-      <c r="I4" s="34"/>
-      <c r="J4" s="44" t="s">
+      <c r="G8" s="47"/>
+      <c r="H8" s="47"/>
+      <c r="I8" s="48"/>
+      <c r="J8" s="46" t="s">
         <v>47</v>
       </c>
-      <c r="K4" s="33"/>
-      <c r="L4" s="34"/>
-      <c r="M4" s="44" t="s">
+      <c r="K8" s="47"/>
+      <c r="L8" s="48"/>
+      <c r="M8" s="46" t="s">
         <v>46</v>
       </c>
-      <c r="N4" s="34"/>
-      <c r="O4" s="38"/>
-      <c r="P4" s="39"/>
-      <c r="Q4" s="39"/>
-      <c r="R4" s="39"/>
-      <c r="S4" s="39"/>
-      <c r="T4" s="39"/>
-      <c r="U4" s="40"/>
-      <c r="V4" s="42"/>
-      <c r="W4" s="30"/>
-      <c r="X4" s="30"/>
-    </row>
-    <row r="5" spans="1:24" ht="114" x14ac:dyDescent="0.2">
-      <c r="A5" s="15" t="s">
+      <c r="N8" s="48"/>
+      <c r="O8" s="52"/>
+      <c r="P8" s="53"/>
+      <c r="Q8" s="53"/>
+      <c r="R8" s="53"/>
+      <c r="S8" s="53"/>
+      <c r="T8" s="53"/>
+      <c r="U8" s="54"/>
+      <c r="V8" s="56"/>
+      <c r="W8" s="42"/>
+      <c r="X8" s="42"/>
+    </row>
+    <row r="9" spans="1:24" ht="114" x14ac:dyDescent="0.2">
+      <c r="A9" s="15" t="s">
         <v>88</v>
       </c>
-      <c r="B5" s="26"/>
-      <c r="C5" s="66"/>
-      <c r="D5" s="31"/>
-      <c r="E5" s="31"/>
-      <c r="F5" s="11" t="s">
+      <c r="B9" s="38"/>
+      <c r="C9" s="40"/>
+      <c r="D9" s="43"/>
+      <c r="E9" s="43"/>
+      <c r="F9" s="11" t="s">
         <v>56</v>
       </c>
-      <c r="G5" s="11" t="s">
+      <c r="G9" s="11" t="s">
         <v>57</v>
       </c>
-      <c r="H5" s="11" t="s">
+      <c r="H9" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="I5" s="11" t="s">
+      <c r="I9" s="11" t="s">
         <v>59</v>
       </c>
-      <c r="J5" s="11" t="s">
+      <c r="J9" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="K5" s="11" t="s">
+      <c r="K9" s="11" t="s">
         <v>61</v>
       </c>
-      <c r="L5" s="11" t="s">
+      <c r="L9" s="11" t="s">
         <v>80</v>
       </c>
-      <c r="M5" s="11" t="s">
+      <c r="M9" s="11" t="s">
         <v>62</v>
       </c>
-      <c r="N5" s="11" t="s">
+      <c r="N9" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="O5" s="11" t="s">
+      <c r="O9" s="11" t="s">
         <v>64</v>
       </c>
-      <c r="P5" s="11" t="s">
+      <c r="P9" s="11" t="s">
         <v>65</v>
       </c>
-      <c r="Q5" s="11" t="s">
+      <c r="Q9" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="R5" s="11" t="s">
+      <c r="R9" s="11" t="s">
         <v>75</v>
       </c>
-      <c r="S5" s="11" t="s">
+      <c r="S9" s="11" t="s">
         <v>76</v>
       </c>
-      <c r="T5" s="11" t="s">
+      <c r="T9" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="U5" s="11" t="s">
+      <c r="U9" s="11" t="s">
         <v>81</v>
       </c>
-      <c r="V5" s="43"/>
-      <c r="W5" s="31"/>
-      <c r="X5" s="31"/>
-    </row>
-    <row r="6" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A6" s="70"/>
-      <c r="B6" s="9"/>
-      <c r="C6" s="9"/>
-      <c r="D6" s="9"/>
-      <c r="E6" s="9"/>
-      <c r="F6" s="9"/>
-      <c r="G6" s="9"/>
-      <c r="H6" s="9"/>
-      <c r="I6" s="9"/>
-      <c r="J6" s="9"/>
-      <c r="K6" s="9"/>
-      <c r="L6" s="9"/>
-      <c r="M6" s="9"/>
-      <c r="N6" s="9"/>
-      <c r="O6" s="9"/>
-      <c r="P6" s="9"/>
-      <c r="Q6" s="9"/>
-      <c r="R6" s="9"/>
-      <c r="S6" s="9"/>
-      <c r="T6" s="18"/>
-      <c r="U6" s="9"/>
-      <c r="V6" s="9"/>
-      <c r="W6" s="9"/>
-      <c r="X6" s="9"/>
-    </row>
-    <row r="7" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A7" s="71"/>
-      <c r="B7" s="9"/>
-      <c r="C7" s="9"/>
-      <c r="D7" s="9"/>
-      <c r="E7" s="9"/>
-      <c r="F7" s="9"/>
-      <c r="G7" s="9"/>
-      <c r="H7" s="9"/>
-      <c r="I7" s="9"/>
-      <c r="J7" s="9"/>
-      <c r="K7" s="9"/>
-      <c r="L7" s="9"/>
-      <c r="M7" s="9"/>
-      <c r="N7" s="9"/>
-      <c r="O7" s="9"/>
-      <c r="P7" s="9"/>
-      <c r="Q7" s="9"/>
-      <c r="R7" s="9"/>
-      <c r="S7" s="9"/>
-      <c r="T7" s="18"/>
-      <c r="U7" s="9"/>
-      <c r="V7" s="9"/>
-      <c r="W7" s="9"/>
-      <c r="X7" s="9"/>
-    </row>
-    <row r="8" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A8" s="71"/>
-      <c r="B8" s="9"/>
-      <c r="C8" s="9"/>
-      <c r="D8" s="9"/>
-      <c r="E8" s="9"/>
-      <c r="F8" s="9"/>
-      <c r="G8" s="9"/>
-      <c r="H8" s="9"/>
-      <c r="I8" s="9"/>
-      <c r="J8" s="9"/>
-      <c r="K8" s="9"/>
-      <c r="L8" s="9"/>
-      <c r="M8" s="9"/>
-      <c r="N8" s="9"/>
-      <c r="O8" s="9"/>
-      <c r="P8" s="9"/>
-      <c r="Q8" s="9"/>
-      <c r="R8" s="9"/>
-      <c r="S8" s="9"/>
-      <c r="T8" s="18"/>
-      <c r="U8" s="9"/>
-      <c r="V8" s="9"/>
-      <c r="W8" s="9"/>
-      <c r="X8" s="9"/>
-    </row>
-    <row r="9" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A9" s="71"/>
-      <c r="B9" s="9"/>
-      <c r="C9" s="9"/>
-      <c r="D9" s="9"/>
-      <c r="E9" s="9"/>
-      <c r="F9" s="9"/>
-      <c r="G9" s="9"/>
-      <c r="H9" s="9"/>
-      <c r="I9" s="9"/>
-      <c r="J9" s="9"/>
-      <c r="K9" s="9"/>
-      <c r="L9" s="9"/>
-      <c r="M9" s="9"/>
-      <c r="N9" s="9"/>
-      <c r="O9" s="9"/>
-      <c r="P9" s="9"/>
-      <c r="Q9" s="9"/>
-      <c r="R9" s="9"/>
-      <c r="S9" s="9"/>
-      <c r="T9" s="18"/>
-      <c r="U9" s="9"/>
-      <c r="V9" s="9"/>
-      <c r="W9" s="9"/>
-      <c r="X9" s="9"/>
+      <c r="V9" s="57"/>
+      <c r="W9" s="43"/>
+      <c r="X9" s="43"/>
     </row>
     <row r="10" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A10" s="71"/>
+      <c r="A10" s="28"/>
       <c r="B10" s="9"/>
       <c r="C10" s="9"/>
       <c r="D10" s="9"/>
@@ -4699,7 +4838,7 @@
       <c r="X10" s="9"/>
     </row>
     <row r="11" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A11" s="71"/>
+      <c r="A11" s="29"/>
       <c r="B11" s="9"/>
       <c r="C11" s="9"/>
       <c r="D11" s="9"/>
@@ -4725,7 +4864,7 @@
       <c r="X11" s="9"/>
     </row>
     <row r="12" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A12" s="71"/>
+      <c r="A12" s="29"/>
       <c r="B12" s="9"/>
       <c r="C12" s="9"/>
       <c r="D12" s="9"/>
@@ -4751,7 +4890,7 @@
       <c r="X12" s="9"/>
     </row>
     <row r="13" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A13" s="71"/>
+      <c r="A13" s="29"/>
       <c r="B13" s="9"/>
       <c r="C13" s="9"/>
       <c r="D13" s="9"/>
@@ -4777,7 +4916,7 @@
       <c r="X13" s="9"/>
     </row>
     <row r="14" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A14" s="71"/>
+      <c r="A14" s="29"/>
       <c r="B14" s="9"/>
       <c r="C14" s="9"/>
       <c r="D14" s="9"/>
@@ -4803,7 +4942,7 @@
       <c r="X14" s="9"/>
     </row>
     <row r="15" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A15" s="71"/>
+      <c r="A15" s="29"/>
       <c r="B15" s="9"/>
       <c r="C15" s="9"/>
       <c r="D15" s="9"/>
@@ -4829,7 +4968,7 @@
       <c r="X15" s="9"/>
     </row>
     <row r="16" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A16" s="71"/>
+      <c r="A16" s="29"/>
       <c r="B16" s="9"/>
       <c r="C16" s="9"/>
       <c r="D16" s="9"/>
@@ -4850,12 +4989,12 @@
       <c r="S16" s="9"/>
       <c r="T16" s="18"/>
       <c r="U16" s="9"/>
-      <c r="V16" s="12"/>
-      <c r="W16" s="12"/>
-      <c r="X16" s="12"/>
+      <c r="V16" s="9"/>
+      <c r="W16" s="9"/>
+      <c r="X16" s="9"/>
     </row>
     <row r="17" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A17" s="71"/>
+      <c r="A17" s="29"/>
       <c r="B17" s="9"/>
       <c r="C17" s="9"/>
       <c r="D17" s="9"/>
@@ -4876,12 +5015,12 @@
       <c r="S17" s="9"/>
       <c r="T17" s="18"/>
       <c r="U17" s="9"/>
-      <c r="V17" s="12"/>
-      <c r="W17" s="12"/>
-      <c r="X17" s="12"/>
+      <c r="V17" s="9"/>
+      <c r="W17" s="9"/>
+      <c r="X17" s="9"/>
     </row>
     <row r="18" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A18" s="72"/>
+      <c r="A18" s="29"/>
       <c r="B18" s="9"/>
       <c r="C18" s="9"/>
       <c r="D18" s="9"/>
@@ -4902,68 +5041,176 @@
       <c r="S18" s="9"/>
       <c r="T18" s="18"/>
       <c r="U18" s="9"/>
-      <c r="V18" s="12"/>
-      <c r="W18" s="12"/>
-      <c r="X18" s="12"/>
-    </row>
-    <row r="29" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A29" s="27" t="s">
+      <c r="V18" s="9"/>
+      <c r="W18" s="9"/>
+      <c r="X18" s="9"/>
+    </row>
+    <row r="19" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A19" s="29"/>
+      <c r="B19" s="9"/>
+      <c r="C19" s="9"/>
+      <c r="D19" s="9"/>
+      <c r="E19" s="9"/>
+      <c r="F19" s="9"/>
+      <c r="G19" s="9"/>
+      <c r="H19" s="9"/>
+      <c r="I19" s="9"/>
+      <c r="J19" s="9"/>
+      <c r="K19" s="9"/>
+      <c r="L19" s="9"/>
+      <c r="M19" s="9"/>
+      <c r="N19" s="9"/>
+      <c r="O19" s="9"/>
+      <c r="P19" s="9"/>
+      <c r="Q19" s="9"/>
+      <c r="R19" s="9"/>
+      <c r="S19" s="9"/>
+      <c r="T19" s="18"/>
+      <c r="U19" s="9"/>
+      <c r="V19" s="9"/>
+      <c r="W19" s="9"/>
+      <c r="X19" s="9"/>
+    </row>
+    <row r="20" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A20" s="29"/>
+      <c r="B20" s="9"/>
+      <c r="C20" s="9"/>
+      <c r="D20" s="9"/>
+      <c r="E20" s="9"/>
+      <c r="F20" s="9"/>
+      <c r="G20" s="9"/>
+      <c r="H20" s="9"/>
+      <c r="I20" s="9"/>
+      <c r="J20" s="9"/>
+      <c r="K20" s="9"/>
+      <c r="L20" s="9"/>
+      <c r="M20" s="9"/>
+      <c r="N20" s="9"/>
+      <c r="O20" s="9"/>
+      <c r="P20" s="9"/>
+      <c r="Q20" s="9"/>
+      <c r="R20" s="9"/>
+      <c r="S20" s="9"/>
+      <c r="T20" s="18"/>
+      <c r="U20" s="9"/>
+      <c r="V20" s="12"/>
+      <c r="W20" s="12"/>
+      <c r="X20" s="12"/>
+    </row>
+    <row r="21" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A21" s="29"/>
+      <c r="B21" s="9"/>
+      <c r="C21" s="9"/>
+      <c r="D21" s="9"/>
+      <c r="E21" s="9"/>
+      <c r="F21" s="9"/>
+      <c r="G21" s="9"/>
+      <c r="H21" s="9"/>
+      <c r="I21" s="9"/>
+      <c r="J21" s="9"/>
+      <c r="K21" s="9"/>
+      <c r="L21" s="9"/>
+      <c r="M21" s="9"/>
+      <c r="N21" s="9"/>
+      <c r="O21" s="9"/>
+      <c r="P21" s="9"/>
+      <c r="Q21" s="9"/>
+      <c r="R21" s="9"/>
+      <c r="S21" s="9"/>
+      <c r="T21" s="18"/>
+      <c r="U21" s="9"/>
+      <c r="V21" s="12"/>
+      <c r="W21" s="12"/>
+      <c r="X21" s="12"/>
+    </row>
+    <row r="22" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A22" s="30"/>
+      <c r="B22" s="9"/>
+      <c r="C22" s="9"/>
+      <c r="D22" s="9"/>
+      <c r="E22" s="9"/>
+      <c r="F22" s="9"/>
+      <c r="G22" s="9"/>
+      <c r="H22" s="9"/>
+      <c r="I22" s="9"/>
+      <c r="J22" s="9"/>
+      <c r="K22" s="9"/>
+      <c r="L22" s="9"/>
+      <c r="M22" s="9"/>
+      <c r="N22" s="9"/>
+      <c r="O22" s="9"/>
+      <c r="P22" s="9"/>
+      <c r="Q22" s="9"/>
+      <c r="R22" s="9"/>
+      <c r="S22" s="9"/>
+      <c r="T22" s="18"/>
+      <c r="U22" s="9"/>
+      <c r="V22" s="12"/>
+      <c r="W22" s="12"/>
+      <c r="X22" s="12"/>
+    </row>
+    <row r="29" spans="1:24" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="30" spans="1:24" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="31" spans="1:24" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="32" spans="1:24" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="33" spans="1:5" ht="18" x14ac:dyDescent="0.2">
+      <c r="A33" s="31" t="s">
         <v>92</v>
       </c>
-      <c r="B29" s="27"/>
-      <c r="C29" s="27"/>
-      <c r="D29" s="27"/>
-      <c r="E29" s="28"/>
-    </row>
-    <row r="30" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A30" s="27"/>
-      <c r="B30" s="27"/>
-      <c r="C30" s="27"/>
-      <c r="D30" s="27"/>
-      <c r="E30" s="28"/>
-    </row>
-    <row r="31" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A31" s="27" t="s">
+      <c r="B33" s="31"/>
+      <c r="C33" s="26"/>
+      <c r="D33" s="26"/>
+      <c r="E33" s="27"/>
+    </row>
+    <row r="34" spans="1:5" ht="18" x14ac:dyDescent="0.2">
+      <c r="A34" s="26"/>
+      <c r="B34" s="26"/>
+      <c r="C34" s="26"/>
+      <c r="D34" s="26"/>
+      <c r="E34" s="27"/>
+    </row>
+    <row r="35" spans="1:5" ht="18" x14ac:dyDescent="0.2">
+      <c r="A35" s="31" t="s">
         <v>91</v>
       </c>
-      <c r="B31" s="27"/>
-      <c r="C31" s="27"/>
-      <c r="D31" s="27"/>
-      <c r="E31" s="28"/>
-    </row>
-    <row r="32" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A32" s="27"/>
-      <c r="B32" s="27"/>
-      <c r="C32" s="27"/>
-      <c r="D32" s="27"/>
-      <c r="E32" s="28"/>
+      <c r="B35" s="31"/>
+      <c r="C35" s="26"/>
+      <c r="D35" s="26"/>
+      <c r="E35" s="27"/>
+    </row>
+    <row r="36" spans="1:5" ht="18" x14ac:dyDescent="0.2">
+      <c r="A36" s="26"/>
+      <c r="B36" s="26"/>
+      <c r="C36" s="26"/>
+      <c r="D36" s="26"/>
+      <c r="E36" s="27"/>
     </row>
   </sheetData>
   <dataConsolidate/>
   <mergeCells count="19">
-    <mergeCell ref="X2:X5"/>
-    <mergeCell ref="F3:N3"/>
-    <mergeCell ref="O3:U4"/>
-    <mergeCell ref="V3:V5"/>
-    <mergeCell ref="F4:I4"/>
-    <mergeCell ref="J4:L4"/>
-    <mergeCell ref="M4:N4"/>
-    <mergeCell ref="W2:W5"/>
-    <mergeCell ref="F2:U2"/>
-    <mergeCell ref="B2:B5"/>
-    <mergeCell ref="A29:D30"/>
-    <mergeCell ref="E29:E30"/>
-    <mergeCell ref="A31:D32"/>
-    <mergeCell ref="E31:E32"/>
-    <mergeCell ref="C2:C5"/>
-    <mergeCell ref="D2:D5"/>
-    <mergeCell ref="E2:E5"/>
-    <mergeCell ref="A6:A18"/>
-    <mergeCell ref="A2:A4"/>
+    <mergeCell ref="M8:N8"/>
+    <mergeCell ref="W6:W9"/>
+    <mergeCell ref="F6:U6"/>
+    <mergeCell ref="E1:U5"/>
+    <mergeCell ref="V1:X5"/>
+    <mergeCell ref="A1:D5"/>
+    <mergeCell ref="A35:B35"/>
+    <mergeCell ref="A33:B33"/>
+    <mergeCell ref="B6:B9"/>
+    <mergeCell ref="C6:C9"/>
+    <mergeCell ref="D6:D9"/>
+    <mergeCell ref="E6:E9"/>
+    <mergeCell ref="A6:A8"/>
+    <mergeCell ref="X6:X9"/>
+    <mergeCell ref="F7:N7"/>
+    <mergeCell ref="O7:U8"/>
+    <mergeCell ref="V7:V9"/>
+    <mergeCell ref="F8:I8"/>
+    <mergeCell ref="J8:L8"/>
   </mergeCells>
-  <conditionalFormatting sqref="U6:U18">
+  <conditionalFormatting sqref="U10:U22">
     <cfRule type="containsText" dxfId="1" priority="1" stopIfTrue="1" operator="containsText" text="SI">
-      <formula>NOT(ISERROR(SEARCH("SI",U6)))</formula>
+      <formula>NOT(ISERROR(SEARCH("SI",U10)))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="2">
       <colorScale>
@@ -4977,13 +5224,8 @@
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.70866141732283472" right="0.59055118110236227" top="1.1578124999999999" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup paperSize="119" scale="47" fitToHeight="0" orientation="landscape" r:id="rId1"/>
+  <pageSetup paperSize="119" fitToHeight="0" orientation="landscape" r:id="rId1"/>
   <headerFooter>
-    <oddHeader>&amp;C&amp;"Arial,Regular"&amp;14&amp;KFF0000SUPERSERVICIO CUATRO CAMINOS S.A DE C.V&amp;K01+000
-&amp;7TÍTULO
-&amp;11MATRIZ DE ASPECTOS E IMPACTOS AMBIENTALES
-&amp;8Revisión Número: 0&amp;R&amp;9CLAVE: F-02-02           
-   &amp;11    FECHA DE EMISIÓN:&amp;KFF000001/03/2019</oddHeader>
     <oddFooter>&amp;R&amp;P DE &amp;N</oddFooter>
   </headerFooter>
   <drawing r:id="rId2"/>
@@ -4995,13 +5237,13 @@
           <x14:formula1>
             <xm:f>'Lista de AA'!$D$3:$D$18</xm:f>
           </x14:formula1>
-          <xm:sqref>D6:D18</xm:sqref>
+          <xm:sqref>D10:D22</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0300-000001000000}">
           <x14:formula1>
             <xm:f>'Lista de AA'!$B$3:$B$8</xm:f>
           </x14:formula1>
-          <xm:sqref>A5</xm:sqref>
+          <xm:sqref>A9</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -5014,7 +5256,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:X32"/>
+  <dimension ref="A1:X36"/>
   <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="31.85546875" style="10" customWidth="1"/>
@@ -5035,278 +5277,310 @@
     <col min="25" max="16384" width="10.85546875" style="10"/>
   </cols>
   <sheetData>
+    <row r="1" spans="1:24" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="35" t="s">
+        <v>98</v>
+      </c>
+      <c r="B1" s="35"/>
+      <c r="C1" s="35"/>
+      <c r="D1" s="35"/>
+      <c r="E1" s="36" t="s">
+        <v>99</v>
+      </c>
+      <c r="F1" s="35"/>
+      <c r="G1" s="35"/>
+      <c r="H1" s="35"/>
+      <c r="I1" s="35"/>
+      <c r="J1" s="35"/>
+      <c r="K1" s="35"/>
+      <c r="L1" s="35"/>
+      <c r="M1" s="35"/>
+      <c r="N1" s="35"/>
+      <c r="O1" s="35"/>
+      <c r="P1" s="35"/>
+      <c r="Q1" s="35"/>
+      <c r="R1" s="35"/>
+      <c r="S1" s="35"/>
+      <c r="T1" s="35"/>
+      <c r="U1" s="35"/>
+      <c r="V1" s="35"/>
+      <c r="W1" s="32" t="s">
+        <v>97</v>
+      </c>
+      <c r="X1" s="33"/>
+    </row>
     <row r="2" spans="1:24" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="67" t="s">
+      <c r="A2" s="35"/>
+      <c r="B2" s="35"/>
+      <c r="C2" s="35"/>
+      <c r="D2" s="35"/>
+      <c r="E2" s="35"/>
+      <c r="F2" s="35"/>
+      <c r="G2" s="35"/>
+      <c r="H2" s="35"/>
+      <c r="I2" s="35"/>
+      <c r="J2" s="35"/>
+      <c r="K2" s="35"/>
+      <c r="L2" s="35"/>
+      <c r="M2" s="35"/>
+      <c r="N2" s="35"/>
+      <c r="O2" s="35"/>
+      <c r="P2" s="35"/>
+      <c r="Q2" s="35"/>
+      <c r="R2" s="35"/>
+      <c r="S2" s="35"/>
+      <c r="T2" s="35"/>
+      <c r="U2" s="35"/>
+      <c r="V2" s="35"/>
+      <c r="W2" s="33"/>
+      <c r="X2" s="33"/>
+    </row>
+    <row r="3" spans="1:24" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="35"/>
+      <c r="B3" s="35"/>
+      <c r="C3" s="35"/>
+      <c r="D3" s="35"/>
+      <c r="E3" s="35"/>
+      <c r="F3" s="35"/>
+      <c r="G3" s="35"/>
+      <c r="H3" s="35"/>
+      <c r="I3" s="35"/>
+      <c r="J3" s="35"/>
+      <c r="K3" s="35"/>
+      <c r="L3" s="35"/>
+      <c r="M3" s="35"/>
+      <c r="N3" s="35"/>
+      <c r="O3" s="35"/>
+      <c r="P3" s="35"/>
+      <c r="Q3" s="35"/>
+      <c r="R3" s="35"/>
+      <c r="S3" s="35"/>
+      <c r="T3" s="35"/>
+      <c r="U3" s="35"/>
+      <c r="V3" s="35"/>
+      <c r="W3" s="33"/>
+      <c r="X3" s="33"/>
+    </row>
+    <row r="4" spans="1:24" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="35"/>
+      <c r="B4" s="35"/>
+      <c r="C4" s="35"/>
+      <c r="D4" s="35"/>
+      <c r="E4" s="35"/>
+      <c r="F4" s="35"/>
+      <c r="G4" s="35"/>
+      <c r="H4" s="35"/>
+      <c r="I4" s="35"/>
+      <c r="J4" s="35"/>
+      <c r="K4" s="35"/>
+      <c r="L4" s="35"/>
+      <c r="M4" s="35"/>
+      <c r="N4" s="35"/>
+      <c r="O4" s="35"/>
+      <c r="P4" s="35"/>
+      <c r="Q4" s="35"/>
+      <c r="R4" s="35"/>
+      <c r="S4" s="35"/>
+      <c r="T4" s="35"/>
+      <c r="U4" s="35"/>
+      <c r="V4" s="35"/>
+      <c r="W4" s="33"/>
+      <c r="X4" s="33"/>
+    </row>
+    <row r="5" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A5" s="35"/>
+      <c r="B5" s="35"/>
+      <c r="C5" s="35"/>
+      <c r="D5" s="35"/>
+      <c r="E5" s="37"/>
+      <c r="F5" s="37"/>
+      <c r="G5" s="37"/>
+      <c r="H5" s="37"/>
+      <c r="I5" s="37"/>
+      <c r="J5" s="37"/>
+      <c r="K5" s="37"/>
+      <c r="L5" s="37"/>
+      <c r="M5" s="37"/>
+      <c r="N5" s="37"/>
+      <c r="O5" s="37"/>
+      <c r="P5" s="37"/>
+      <c r="Q5" s="37"/>
+      <c r="R5" s="37"/>
+      <c r="S5" s="37"/>
+      <c r="T5" s="37"/>
+      <c r="U5" s="37"/>
+      <c r="V5" s="37"/>
+      <c r="W5" s="34"/>
+      <c r="X5" s="34"/>
+    </row>
+    <row r="6" spans="1:24" ht="15" x14ac:dyDescent="0.2">
+      <c r="A6" s="44" t="s">
         <v>32</v>
       </c>
-      <c r="B2" s="26" t="s">
+      <c r="B6" s="38" t="s">
         <v>54</v>
       </c>
-      <c r="C2" s="65" t="s">
+      <c r="C6" s="39" t="s">
         <v>53</v>
       </c>
-      <c r="D2" s="29" t="s">
+      <c r="D6" s="41" t="s">
         <v>50</v>
       </c>
-      <c r="E2" s="29" t="s">
+      <c r="E6" s="41" t="s">
         <v>48</v>
       </c>
-      <c r="F2" s="69" t="s">
+      <c r="F6" s="58" t="s">
         <v>55</v>
       </c>
-      <c r="G2" s="45"/>
-      <c r="H2" s="45"/>
-      <c r="I2" s="45"/>
-      <c r="J2" s="45"/>
-      <c r="K2" s="45"/>
-      <c r="L2" s="45"/>
-      <c r="M2" s="45"/>
-      <c r="N2" s="45"/>
-      <c r="O2" s="45"/>
-      <c r="P2" s="45"/>
-      <c r="Q2" s="45"/>
-      <c r="R2" s="45"/>
-      <c r="S2" s="45"/>
-      <c r="T2" s="45"/>
-      <c r="U2" s="46"/>
-      <c r="V2" s="16"/>
-      <c r="W2" s="29" t="s">
+      <c r="G6" s="59"/>
+      <c r="H6" s="59"/>
+      <c r="I6" s="59"/>
+      <c r="J6" s="59"/>
+      <c r="K6" s="59"/>
+      <c r="L6" s="59"/>
+      <c r="M6" s="59"/>
+      <c r="N6" s="59"/>
+      <c r="O6" s="59"/>
+      <c r="P6" s="59"/>
+      <c r="Q6" s="59"/>
+      <c r="R6" s="59"/>
+      <c r="S6" s="59"/>
+      <c r="T6" s="59"/>
+      <c r="U6" s="60"/>
+      <c r="V6" s="16"/>
+      <c r="W6" s="41" t="s">
         <v>71</v>
       </c>
-      <c r="X2" s="29" t="s">
+      <c r="X6" s="41" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="3" spans="1:24" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="67"/>
-      <c r="B3" s="26"/>
-      <c r="C3" s="65"/>
-      <c r="D3" s="30"/>
-      <c r="E3" s="30"/>
-      <c r="F3" s="44" t="s">
+    <row r="7" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A7" s="44"/>
+      <c r="B7" s="38"/>
+      <c r="C7" s="39"/>
+      <c r="D7" s="42"/>
+      <c r="E7" s="42"/>
+      <c r="F7" s="46" t="s">
         <v>49</v>
       </c>
-      <c r="G3" s="33"/>
-      <c r="H3" s="33"/>
-      <c r="I3" s="33"/>
-      <c r="J3" s="33"/>
-      <c r="K3" s="33"/>
-      <c r="L3" s="33"/>
-      <c r="M3" s="33"/>
-      <c r="N3" s="34"/>
-      <c r="O3" s="35" t="s">
+      <c r="G7" s="47"/>
+      <c r="H7" s="47"/>
+      <c r="I7" s="47"/>
+      <c r="J7" s="47"/>
+      <c r="K7" s="47"/>
+      <c r="L7" s="47"/>
+      <c r="M7" s="47"/>
+      <c r="N7" s="48"/>
+      <c r="O7" s="49" t="s">
         <v>44</v>
       </c>
-      <c r="P3" s="36"/>
-      <c r="Q3" s="36"/>
-      <c r="R3" s="36"/>
-      <c r="S3" s="36"/>
-      <c r="T3" s="36"/>
-      <c r="U3" s="37"/>
-      <c r="V3" s="41" t="s">
+      <c r="P7" s="50"/>
+      <c r="Q7" s="50"/>
+      <c r="R7" s="50"/>
+      <c r="S7" s="50"/>
+      <c r="T7" s="50"/>
+      <c r="U7" s="51"/>
+      <c r="V7" s="55" t="s">
         <v>67</v>
       </c>
-      <c r="W3" s="30"/>
-      <c r="X3" s="30"/>
-    </row>
-    <row r="4" spans="1:24" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="68"/>
-      <c r="B4" s="26"/>
-      <c r="C4" s="65"/>
-      <c r="D4" s="30"/>
-      <c r="E4" s="30"/>
-      <c r="F4" s="44" t="s">
+      <c r="W7" s="42"/>
+      <c r="X7" s="42"/>
+    </row>
+    <row r="8" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A8" s="45"/>
+      <c r="B8" s="38"/>
+      <c r="C8" s="39"/>
+      <c r="D8" s="42"/>
+      <c r="E8" s="42"/>
+      <c r="F8" s="46" t="s">
         <v>45</v>
       </c>
-      <c r="G4" s="33"/>
-      <c r="H4" s="33"/>
-      <c r="I4" s="34"/>
-      <c r="J4" s="44" t="s">
+      <c r="G8" s="47"/>
+      <c r="H8" s="47"/>
+      <c r="I8" s="48"/>
+      <c r="J8" s="46" t="s">
         <v>47</v>
       </c>
-      <c r="K4" s="33"/>
-      <c r="L4" s="34"/>
-      <c r="M4" s="44" t="s">
+      <c r="K8" s="47"/>
+      <c r="L8" s="48"/>
+      <c r="M8" s="46" t="s">
         <v>46</v>
       </c>
-      <c r="N4" s="34"/>
-      <c r="O4" s="38"/>
-      <c r="P4" s="39"/>
-      <c r="Q4" s="39"/>
-      <c r="R4" s="39"/>
-      <c r="S4" s="39"/>
-      <c r="T4" s="39"/>
-      <c r="U4" s="40"/>
-      <c r="V4" s="42"/>
-      <c r="W4" s="30"/>
-      <c r="X4" s="30"/>
-    </row>
-    <row r="5" spans="1:24" ht="114" x14ac:dyDescent="0.2">
-      <c r="A5" s="15" t="s">
+      <c r="N8" s="48"/>
+      <c r="O8" s="52"/>
+      <c r="P8" s="53"/>
+      <c r="Q8" s="53"/>
+      <c r="R8" s="53"/>
+      <c r="S8" s="53"/>
+      <c r="T8" s="53"/>
+      <c r="U8" s="54"/>
+      <c r="V8" s="56"/>
+      <c r="W8" s="42"/>
+      <c r="X8" s="42"/>
+    </row>
+    <row r="9" spans="1:24" ht="114" x14ac:dyDescent="0.2">
+      <c r="A9" s="15" t="s">
         <v>89</v>
       </c>
-      <c r="B5" s="26"/>
-      <c r="C5" s="66"/>
-      <c r="D5" s="31"/>
-      <c r="E5" s="31"/>
-      <c r="F5" s="11" t="s">
+      <c r="B9" s="38"/>
+      <c r="C9" s="40"/>
+      <c r="D9" s="43"/>
+      <c r="E9" s="43"/>
+      <c r="F9" s="11" t="s">
         <v>56</v>
       </c>
-      <c r="G5" s="11" t="s">
+      <c r="G9" s="11" t="s">
         <v>57</v>
       </c>
-      <c r="H5" s="11" t="s">
+      <c r="H9" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="I5" s="11" t="s">
+      <c r="I9" s="11" t="s">
         <v>59</v>
       </c>
-      <c r="J5" s="11" t="s">
+      <c r="J9" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="K5" s="11" t="s">
+      <c r="K9" s="11" t="s">
         <v>61</v>
       </c>
-      <c r="L5" s="11" t="s">
+      <c r="L9" s="11" t="s">
         <v>80</v>
       </c>
-      <c r="M5" s="11" t="s">
+      <c r="M9" s="11" t="s">
         <v>62</v>
       </c>
-      <c r="N5" s="11" t="s">
+      <c r="N9" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="O5" s="11" t="s">
+      <c r="O9" s="11" t="s">
         <v>64</v>
       </c>
-      <c r="P5" s="11" t="s">
+      <c r="P9" s="11" t="s">
         <v>65</v>
       </c>
-      <c r="Q5" s="11" t="s">
+      <c r="Q9" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="R5" s="11" t="s">
+      <c r="R9" s="11" t="s">
         <v>75</v>
       </c>
-      <c r="S5" s="11" t="s">
+      <c r="S9" s="11" t="s">
         <v>76</v>
       </c>
-      <c r="T5" s="11" t="s">
+      <c r="T9" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="U5" s="11" t="s">
+      <c r="U9" s="11" t="s">
         <v>81</v>
       </c>
-      <c r="V5" s="43"/>
-      <c r="W5" s="31"/>
-      <c r="X5" s="31"/>
-    </row>
-    <row r="6" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A6" s="70"/>
-      <c r="B6" s="9"/>
-      <c r="C6" s="9"/>
-      <c r="D6" s="9"/>
-      <c r="E6" s="9"/>
-      <c r="F6" s="9"/>
-      <c r="G6" s="9"/>
-      <c r="H6" s="9"/>
-      <c r="I6" s="9"/>
-      <c r="J6" s="9"/>
-      <c r="K6" s="9"/>
-      <c r="L6" s="9"/>
-      <c r="M6" s="9"/>
-      <c r="N6" s="9"/>
-      <c r="O6" s="9"/>
-      <c r="P6" s="9"/>
-      <c r="Q6" s="9"/>
-      <c r="R6" s="9"/>
-      <c r="S6" s="9"/>
-      <c r="T6" s="18"/>
-      <c r="U6" s="9"/>
-      <c r="V6" s="9"/>
-      <c r="W6" s="9"/>
-      <c r="X6" s="9"/>
-    </row>
-    <row r="7" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A7" s="71"/>
-      <c r="B7" s="9"/>
-      <c r="C7" s="9"/>
-      <c r="D7" s="9"/>
-      <c r="E7" s="9"/>
-      <c r="F7" s="9"/>
-      <c r="G7" s="9"/>
-      <c r="H7" s="9"/>
-      <c r="I7" s="9"/>
-      <c r="J7" s="9"/>
-      <c r="K7" s="9"/>
-      <c r="L7" s="9"/>
-      <c r="M7" s="9"/>
-      <c r="N7" s="9"/>
-      <c r="O7" s="9"/>
-      <c r="P7" s="9"/>
-      <c r="Q7" s="9"/>
-      <c r="R7" s="9"/>
-      <c r="S7" s="9"/>
-      <c r="T7" s="18"/>
-      <c r="U7" s="9"/>
-      <c r="V7" s="9"/>
-      <c r="W7" s="9"/>
-      <c r="X7" s="9"/>
-    </row>
-    <row r="8" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A8" s="71"/>
-      <c r="B8" s="9"/>
-      <c r="C8" s="9"/>
-      <c r="D8" s="9"/>
-      <c r="E8" s="9"/>
-      <c r="F8" s="9"/>
-      <c r="G8" s="9"/>
-      <c r="H8" s="9"/>
-      <c r="I8" s="9"/>
-      <c r="J8" s="9"/>
-      <c r="K8" s="9"/>
-      <c r="L8" s="9"/>
-      <c r="M8" s="9"/>
-      <c r="N8" s="9"/>
-      <c r="O8" s="9"/>
-      <c r="P8" s="9"/>
-      <c r="Q8" s="9"/>
-      <c r="R8" s="9"/>
-      <c r="S8" s="9"/>
-      <c r="T8" s="18"/>
-      <c r="U8" s="9"/>
-      <c r="V8" s="9"/>
-      <c r="W8" s="9"/>
-      <c r="X8" s="9"/>
-    </row>
-    <row r="9" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A9" s="71"/>
-      <c r="B9" s="9"/>
-      <c r="C9" s="9"/>
-      <c r="D9" s="9"/>
-      <c r="E9" s="9"/>
-      <c r="F9" s="9"/>
-      <c r="G9" s="9"/>
-      <c r="H9" s="9"/>
-      <c r="I9" s="9"/>
-      <c r="J9" s="9"/>
-      <c r="K9" s="9"/>
-      <c r="L9" s="9"/>
-      <c r="M9" s="9"/>
-      <c r="N9" s="9"/>
-      <c r="O9" s="9"/>
-      <c r="P9" s="9"/>
-      <c r="Q9" s="9"/>
-      <c r="R9" s="9"/>
-      <c r="S9" s="9"/>
-      <c r="T9" s="18"/>
-      <c r="U9" s="9"/>
-      <c r="V9" s="9"/>
-      <c r="W9" s="9"/>
-      <c r="X9" s="9"/>
+      <c r="V9" s="57"/>
+      <c r="W9" s="43"/>
+      <c r="X9" s="43"/>
     </row>
     <row r="10" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A10" s="71"/>
+      <c r="A10" s="28"/>
       <c r="B10" s="9"/>
       <c r="C10" s="9"/>
       <c r="D10" s="9"/>
@@ -5332,7 +5606,7 @@
       <c r="X10" s="9"/>
     </row>
     <row r="11" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A11" s="71"/>
+      <c r="A11" s="29"/>
       <c r="B11" s="9"/>
       <c r="C11" s="9"/>
       <c r="D11" s="9"/>
@@ -5358,7 +5632,7 @@
       <c r="X11" s="9"/>
     </row>
     <row r="12" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A12" s="71"/>
+      <c r="A12" s="29"/>
       <c r="B12" s="9"/>
       <c r="C12" s="9"/>
       <c r="D12" s="9"/>
@@ -5384,7 +5658,7 @@
       <c r="X12" s="9"/>
     </row>
     <row r="13" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A13" s="71"/>
+      <c r="A13" s="29"/>
       <c r="B13" s="9"/>
       <c r="C13" s="9"/>
       <c r="D13" s="9"/>
@@ -5410,7 +5684,7 @@
       <c r="X13" s="9"/>
     </row>
     <row r="14" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A14" s="71"/>
+      <c r="A14" s="29"/>
       <c r="B14" s="9"/>
       <c r="C14" s="9"/>
       <c r="D14" s="9"/>
@@ -5436,7 +5710,7 @@
       <c r="X14" s="9"/>
     </row>
     <row r="15" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A15" s="71"/>
+      <c r="A15" s="29"/>
       <c r="B15" s="9"/>
       <c r="C15" s="9"/>
       <c r="D15" s="9"/>
@@ -5462,7 +5736,7 @@
       <c r="X15" s="9"/>
     </row>
     <row r="16" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A16" s="71"/>
+      <c r="A16" s="29"/>
       <c r="B16" s="9"/>
       <c r="C16" s="9"/>
       <c r="D16" s="9"/>
@@ -5483,12 +5757,12 @@
       <c r="S16" s="9"/>
       <c r="T16" s="18"/>
       <c r="U16" s="9"/>
-      <c r="V16" s="12"/>
-      <c r="W16" s="12"/>
-      <c r="X16" s="12"/>
+      <c r="V16" s="9"/>
+      <c r="W16" s="9"/>
+      <c r="X16" s="9"/>
     </row>
     <row r="17" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A17" s="71"/>
+      <c r="A17" s="29"/>
       <c r="B17" s="9"/>
       <c r="C17" s="9"/>
       <c r="D17" s="9"/>
@@ -5509,12 +5783,12 @@
       <c r="S17" s="9"/>
       <c r="T17" s="18"/>
       <c r="U17" s="9"/>
-      <c r="V17" s="12"/>
-      <c r="W17" s="12"/>
-      <c r="X17" s="12"/>
+      <c r="V17" s="9"/>
+      <c r="W17" s="9"/>
+      <c r="X17" s="9"/>
     </row>
     <row r="18" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A18" s="72"/>
+      <c r="A18" s="29"/>
       <c r="B18" s="9"/>
       <c r="C18" s="9"/>
       <c r="D18" s="9"/>
@@ -5535,68 +5809,176 @@
       <c r="S18" s="9"/>
       <c r="T18" s="18"/>
       <c r="U18" s="9"/>
-      <c r="V18" s="12"/>
-      <c r="W18" s="12"/>
-      <c r="X18" s="12"/>
-    </row>
-    <row r="29" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A29" s="27" t="s">
+      <c r="V18" s="9"/>
+      <c r="W18" s="9"/>
+      <c r="X18" s="9"/>
+    </row>
+    <row r="19" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A19" s="29"/>
+      <c r="B19" s="9"/>
+      <c r="C19" s="9"/>
+      <c r="D19" s="9"/>
+      <c r="E19" s="9"/>
+      <c r="F19" s="9"/>
+      <c r="G19" s="9"/>
+      <c r="H19" s="9"/>
+      <c r="I19" s="9"/>
+      <c r="J19" s="9"/>
+      <c r="K19" s="9"/>
+      <c r="L19" s="9"/>
+      <c r="M19" s="9"/>
+      <c r="N19" s="9"/>
+      <c r="O19" s="9"/>
+      <c r="P19" s="9"/>
+      <c r="Q19" s="9"/>
+      <c r="R19" s="9"/>
+      <c r="S19" s="9"/>
+      <c r="T19" s="18"/>
+      <c r="U19" s="9"/>
+      <c r="V19" s="9"/>
+      <c r="W19" s="9"/>
+      <c r="X19" s="9"/>
+    </row>
+    <row r="20" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A20" s="29"/>
+      <c r="B20" s="9"/>
+      <c r="C20" s="9"/>
+      <c r="D20" s="9"/>
+      <c r="E20" s="9"/>
+      <c r="F20" s="9"/>
+      <c r="G20" s="9"/>
+      <c r="H20" s="9"/>
+      <c r="I20" s="9"/>
+      <c r="J20" s="9"/>
+      <c r="K20" s="9"/>
+      <c r="L20" s="9"/>
+      <c r="M20" s="9"/>
+      <c r="N20" s="9"/>
+      <c r="O20" s="9"/>
+      <c r="P20" s="9"/>
+      <c r="Q20" s="9"/>
+      <c r="R20" s="9"/>
+      <c r="S20" s="9"/>
+      <c r="T20" s="18"/>
+      <c r="U20" s="9"/>
+      <c r="V20" s="12"/>
+      <c r="W20" s="12"/>
+      <c r="X20" s="12"/>
+    </row>
+    <row r="21" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A21" s="29"/>
+      <c r="B21" s="9"/>
+      <c r="C21" s="9"/>
+      <c r="D21" s="9"/>
+      <c r="E21" s="9"/>
+      <c r="F21" s="9"/>
+      <c r="G21" s="9"/>
+      <c r="H21" s="9"/>
+      <c r="I21" s="9"/>
+      <c r="J21" s="9"/>
+      <c r="K21" s="9"/>
+      <c r="L21" s="9"/>
+      <c r="M21" s="9"/>
+      <c r="N21" s="9"/>
+      <c r="O21" s="9"/>
+      <c r="P21" s="9"/>
+      <c r="Q21" s="9"/>
+      <c r="R21" s="9"/>
+      <c r="S21" s="9"/>
+      <c r="T21" s="18"/>
+      <c r="U21" s="9"/>
+      <c r="V21" s="12"/>
+      <c r="W21" s="12"/>
+      <c r="X21" s="12"/>
+    </row>
+    <row r="22" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A22" s="30"/>
+      <c r="B22" s="9"/>
+      <c r="C22" s="9"/>
+      <c r="D22" s="9"/>
+      <c r="E22" s="9"/>
+      <c r="F22" s="9"/>
+      <c r="G22" s="9"/>
+      <c r="H22" s="9"/>
+      <c r="I22" s="9"/>
+      <c r="J22" s="9"/>
+      <c r="K22" s="9"/>
+      <c r="L22" s="9"/>
+      <c r="M22" s="9"/>
+      <c r="N22" s="9"/>
+      <c r="O22" s="9"/>
+      <c r="P22" s="9"/>
+      <c r="Q22" s="9"/>
+      <c r="R22" s="9"/>
+      <c r="S22" s="9"/>
+      <c r="T22" s="18"/>
+      <c r="U22" s="9"/>
+      <c r="V22" s="12"/>
+      <c r="W22" s="12"/>
+      <c r="X22" s="12"/>
+    </row>
+    <row r="29" spans="1:24" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="30" spans="1:24" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="31" spans="1:24" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="32" spans="1:24" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="33" spans="1:5" ht="18" x14ac:dyDescent="0.2">
+      <c r="A33" s="31" t="s">
         <v>92</v>
       </c>
-      <c r="B29" s="27"/>
-      <c r="C29" s="27"/>
-      <c r="D29" s="27"/>
-      <c r="E29" s="28"/>
-    </row>
-    <row r="30" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A30" s="27"/>
-      <c r="B30" s="27"/>
-      <c r="C30" s="27"/>
-      <c r="D30" s="27"/>
-      <c r="E30" s="28"/>
-    </row>
-    <row r="31" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A31" s="27" t="s">
+      <c r="B33" s="31"/>
+      <c r="C33" s="26"/>
+      <c r="D33" s="26"/>
+      <c r="E33" s="27"/>
+    </row>
+    <row r="34" spans="1:5" ht="18" x14ac:dyDescent="0.2">
+      <c r="A34" s="26"/>
+      <c r="B34" s="26"/>
+      <c r="C34" s="26"/>
+      <c r="D34" s="26"/>
+      <c r="E34" s="27"/>
+    </row>
+    <row r="35" spans="1:5" ht="18" x14ac:dyDescent="0.2">
+      <c r="A35" s="31" t="s">
         <v>91</v>
       </c>
-      <c r="B31" s="27"/>
-      <c r="C31" s="27"/>
-      <c r="D31" s="27"/>
-      <c r="E31" s="28"/>
-    </row>
-    <row r="32" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A32" s="27"/>
-      <c r="B32" s="27"/>
-      <c r="C32" s="27"/>
-      <c r="D32" s="27"/>
-      <c r="E32" s="28"/>
+      <c r="B35" s="31"/>
+      <c r="C35" s="26"/>
+      <c r="D35" s="26"/>
+      <c r="E35" s="27"/>
+    </row>
+    <row r="36" spans="1:5" ht="18" x14ac:dyDescent="0.2">
+      <c r="A36" s="26"/>
+      <c r="B36" s="26"/>
+      <c r="C36" s="26"/>
+      <c r="D36" s="26"/>
+      <c r="E36" s="27"/>
     </row>
   </sheetData>
   <dataConsolidate/>
   <mergeCells count="19">
-    <mergeCell ref="X2:X5"/>
-    <mergeCell ref="F3:N3"/>
-    <mergeCell ref="O3:U4"/>
-    <mergeCell ref="V3:V5"/>
-    <mergeCell ref="F4:I4"/>
-    <mergeCell ref="J4:L4"/>
-    <mergeCell ref="M4:N4"/>
-    <mergeCell ref="W2:W5"/>
-    <mergeCell ref="F2:U2"/>
-    <mergeCell ref="B2:B5"/>
-    <mergeCell ref="A29:D30"/>
-    <mergeCell ref="E29:E30"/>
-    <mergeCell ref="A31:D32"/>
-    <mergeCell ref="E31:E32"/>
-    <mergeCell ref="C2:C5"/>
-    <mergeCell ref="D2:D5"/>
-    <mergeCell ref="E2:E5"/>
-    <mergeCell ref="A6:A18"/>
-    <mergeCell ref="A2:A4"/>
+    <mergeCell ref="M8:N8"/>
+    <mergeCell ref="W6:W9"/>
+    <mergeCell ref="F6:U6"/>
+    <mergeCell ref="A33:B33"/>
+    <mergeCell ref="A35:B35"/>
+    <mergeCell ref="W1:X5"/>
+    <mergeCell ref="A1:D5"/>
+    <mergeCell ref="E1:V5"/>
+    <mergeCell ref="B6:B9"/>
+    <mergeCell ref="C6:C9"/>
+    <mergeCell ref="D6:D9"/>
+    <mergeCell ref="E6:E9"/>
+    <mergeCell ref="A6:A8"/>
+    <mergeCell ref="X6:X9"/>
+    <mergeCell ref="F7:N7"/>
+    <mergeCell ref="O7:U8"/>
+    <mergeCell ref="V7:V9"/>
+    <mergeCell ref="F8:I8"/>
+    <mergeCell ref="J8:L8"/>
   </mergeCells>
-  <conditionalFormatting sqref="U6:U18">
+  <conditionalFormatting sqref="U10:U22">
     <cfRule type="containsText" dxfId="0" priority="1" stopIfTrue="1" operator="containsText" text="SI">
-      <formula>NOT(ISERROR(SEARCH("SI",U6)))</formula>
+      <formula>NOT(ISERROR(SEARCH("SI",U10)))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="2">
       <colorScale>
@@ -5610,32 +5992,28 @@
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.70866141732283472" right="0.59055118110236227" top="1.1842261904761904" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup paperSize="119" scale="46" fitToHeight="0" orientation="landscape" r:id="rId1"/>
+  <pageSetup paperSize="119" fitToHeight="0" orientation="landscape" r:id="rId1"/>
   <headerFooter>
-    <oddHeader>&amp;L
-&amp;C&amp;"Arial,Negrita"&amp;14&amp;KFF0000SUPERSERVICIO CUATRO CAMINOS S.A DE C.V&amp;K000000
-&amp;7TÍTULO
-&amp;11Matriz de Identificación de Aspectos Ambientales 
-&amp;"Arial,Normal"&amp;8Revisión Número: 0&amp;R&amp;9CLAVE: F-02-02           
-  &amp;11     FECHA DE EMISIÓN:&amp;KFF000001/03/2019</oddHeader>
+    <oddHeader xml:space="preserve">&amp;L
+</oddHeader>
     <oddFooter>&amp;R&amp;P DE &amp;N</oddFooter>
   </headerFooter>
   <drawing r:id="rId2"/>
   <legacyDrawing r:id="rId3"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" disablePrompts="1" count="2">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0400-000000000000}">
           <x14:formula1>
             <xm:f>'Lista de AA'!$B$3:$B$8</xm:f>
           </x14:formula1>
-          <xm:sqref>A5</xm:sqref>
+          <xm:sqref>A9</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0400-000001000000}">
           <x14:formula1>
             <xm:f>'Lista de AA'!$D$3:$D$18</xm:f>
           </x14:formula1>
-          <xm:sqref>D6:D18</xm:sqref>
+          <xm:sqref>D10:D22</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>

</xml_diff>